<commit_message>
Cash flow: Complete AV labour hold released and paid 8 Oct
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141HuBtr9dZXPeYR1jN9h28
</commit_message>
<xml_diff>
--- a/cashflow/CTS Cash Flow Forecast - 12102026.xlsx
+++ b/cashflow/CTS Cash Flow Forecast - 12102026.xlsx
@@ -1135,27 +1135,27 @@
       </c>
       <c r="F10" s="119">
         <f>IF(E$8=1,E59,D58)</f>
-        <v>300315.52999999997</v>
+        <v>261282.50999999998</v>
       </c>
       <c r="G10" s="119">
         <f>F10</f>
-        <v>300315.52999999997</v>
+        <v>261282.50999999998</v>
       </c>
       <c r="H10" s="119">
         <f>IF(G$8=1,G59,F58)</f>
-        <v>534919.8166666667</v>
+        <v>495886.79666666663</v>
       </c>
       <c r="I10" s="119">
         <f>H10</f>
-        <v>534919.8166666667</v>
+        <v>495886.79666666663</v>
       </c>
       <c r="J10" s="119">
         <f>IF(I$8=1,I59,H58)</f>
-        <v>269953.74933333334</v>
+        <v>230920.72933333332</v>
       </c>
       <c r="K10" s="119">
         <f>J10</f>
-        <v>269953.74933333334</v>
+        <v>230920.72933333332</v>
       </c>
       <c r="L10" s="119">
         <f>B10</f>
@@ -1716,11 +1716,11 @@
       </c>
       <c r="D27" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Equipment purchases")+Assumptions!$B$29/5</f>
-        <v>4000</v>
+        <v>43033.020000000004</v>
       </c>
       <c r="E27" s="121">
-        <f>ROUND(28736.64*1.1,2)</f>
-        <v>31610.3</v>
+        <f>ROUND(28736.64*1.1,2)+39033.02</f>
+        <v>70643.31999999999</v>
       </c>
       <c r="F27" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Equipment purchases")+Assumptions!$B$29/5</f>
@@ -1739,11 +1739,11 @@
       <c r="K27" s="121" t="n"/>
       <c r="L27" s="120">
         <f>SUM(B27,D27,F27,H27,J27)</f>
-        <v>201453.61000000002</v>
+        <v>240486.63000000003</v>
       </c>
       <c r="M27" s="120">
         <f>SUM(C27,E27,G27,I27,K27)</f>
-        <v>170696.53</v>
+        <v>209729.55</v>
       </c>
       <c r="N27" s="120">
         <f>(C27-B27)*C$8+(E27-D27)*E$8+(G27-F27)*G$8+(I27-H27)*I$8+(K27-J27)*K$8</f>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="O27" s="108" t="inlineStr">
         <is>
-          <t>139k was paid on the 29/09/2026. Remittance (Complete AV) table  under GC approvals was send on the 29/09. Week 2 to 12 Oct: LiveU SDI/modems $26,004 plus small items ($28,737 ex GST per Xero cash P&amp;L).</t>
+          <t>139k was paid on the 29/09/2026. Remittance (Complete AV) table  under GC approvals was send on the 29/09. Week 2 to 12 Oct: LiveU SDI/modems $26,004 plus small items ($28,737 ex GST per Xero cash P&amp;L). Complete AV labour and programming $39,033.02 was released and paid 8 Oct - whole bill now paid.</t>
         </is>
       </c>
     </row>
@@ -1979,11 +1979,11 @@
       </c>
       <c r="D32" s="123">
         <f>D27+D28+D29+D30+D31</f>
-        <v>25112.04</v>
+        <v>64145.060000000005</v>
       </c>
       <c r="E32" s="123">
         <f>E27+E28+E29+E30+E31</f>
-        <v>78843.94</v>
+        <v>117876.95999999999</v>
       </c>
       <c r="F32" s="123">
         <f>F27+F28+F29+F30+F31</f>
@@ -2011,11 +2011,11 @@
       </c>
       <c r="L32" s="123">
         <f>L27+L28+L29+L30+L31</f>
-        <v>319008.68</v>
+        <v>358041.7</v>
       </c>
       <c r="M32" s="123">
         <f>M27+M28+M29+M30+M31</f>
-        <v>217930.16999999998</v>
+        <v>256963.18999999997</v>
       </c>
       <c r="N32" s="123">
         <f>N27+N28+N29+N30+N31</f>
@@ -2914,11 +2914,11 @@
       </c>
       <c r="D55" s="122">
         <f>D24+D32+D49+D53</f>
-        <v>201076.97</v>
+        <v>240109.99</v>
       </c>
       <c r="E55" s="122">
         <f>E24+E32+E49+E53</f>
-        <v>80029.05</v>
+        <v>119062.06999999999</v>
       </c>
       <c r="F55" s="122">
         <f>F24+F32+F49+F66</f>
@@ -2946,11 +2946,11 @@
       </c>
       <c r="L55" s="122">
         <f>L24+L32+L49+L53</f>
-        <v>804956.3139999999</v>
+        <v>843989.3339999999</v>
       </c>
       <c r="M55" s="122">
         <f>M24+M32+M49+M53</f>
-        <v>219360.87999999998</v>
+        <v>258393.89999999997</v>
       </c>
       <c r="N55" s="122">
         <f>N24+N32+N49+N53</f>
@@ -2974,11 +2974,11 @@
       </c>
       <c r="D57" s="122">
         <f>D15-D55</f>
-        <v>-58380.70000000001</v>
+        <v>-97413.72</v>
       </c>
       <c r="E57" s="122">
         <f>E15-E55</f>
-        <v>63173.220000000016</v>
+        <v>24140.200000000026</v>
       </c>
       <c r="F57" s="122">
         <f>F15-F68</f>
@@ -3006,11 +3006,11 @@
       </c>
       <c r="L57" s="122">
         <f>L15-L55</f>
-        <v>-187968.23400000005</v>
+        <v>-227001.25400000007</v>
       </c>
       <c r="M57" s="122">
         <f>M15-M55</f>
-        <v>64016.99000000002</v>
+        <v>24983.97000000003</v>
       </c>
       <c r="N57" s="122">
         <f>N15-N55</f>
@@ -3034,7 +3034,7 @@
       </c>
       <c r="D58" s="125">
         <f>D10+D57</f>
-        <v>300315.52999999997</v>
+        <v>261282.50999999998</v>
       </c>
       <c r="E58" s="125" t="str">
         <f>IF(E$8=1,E10+E57,"")</f>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="F58" s="125">
         <f>F10+F57</f>
-        <v>534919.8166666667</v>
+        <v>495886.79666666663</v>
       </c>
       <c r="G58" s="125" t="str">
         <f>IF(G$8=1,G10+G57,"")</f>
@@ -3050,7 +3050,7 @@
       </c>
       <c r="H58" s="125">
         <f>H10+H57</f>
-        <v>269953.74933333334</v>
+        <v>230920.72933333332</v>
       </c>
       <c r="I58" s="125" t="str">
         <f>IF(I$8=1,I10+I57,"")</f>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="J58" s="125">
         <f>J10+J57</f>
-        <v>309772.966</v>
+        <v>270739.946</v>
       </c>
       <c r="K58" s="125" t="str">
         <f>IF(K$8=1,K10+K57,"")</f>
@@ -3066,7 +3066,7 @@
       </c>
       <c r="L58" s="125">
         <f>J58</f>
-        <v>309772.966</v>
+        <v>270739.946</v>
       </c>
       <c r="M58" s="125">
         <f>IF(K$8=1,K58,IF(I$8=1,I58,IF(G$8=1,G58,IF(E$8=1,E58,IF(C$8=1,C58,"")))))</f>
@@ -3208,19 +3208,19 @@
       </c>
       <c r="D64" s="127">
         <f>IF(Payroll!$I$5=0,0,D58/(Payroll!$I$5/2))</f>
-        <v>6.032370440302104</v>
+        <v>5.248322955166318</v>
       </c>
       <c r="F64" s="127">
         <f>IF(Payroll!$I$5=0,0,F58/(Payroll!$I$5/2))</f>
-        <v>10.744813929508812</v>
+        <v>9.960766444373023</v>
       </c>
       <c r="H64" s="127">
         <f>IF(Payroll!$I$5=0,0,H58/(Payroll!$I$5/2))</f>
-        <v>5.422500187476565</v>
+        <v>4.638452702340778</v>
       </c>
       <c r="J64" s="127">
         <f>IF(Payroll!$I$5=0,0,J58/(Payroll!$I$5/2))</f>
-        <v>6.2223398280572075</v>
+        <v>5.438292342921421</v>
       </c>
       <c r="O64" s="108" t="n"/>
     </row>
@@ -3248,11 +3248,11 @@
       </c>
       <c r="L66" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$G$19:$G$75,"&gt;"&amp;Assumptions!$C$48)</f>
-        <v>69117.8</v>
+        <v>30084.780000000002</v>
       </c>
       <c r="O66" s="108" t="inlineStr">
         <is>
-          <t>Complete AV labour $41,956 (held for Aware sign off), Oct rent, Oct mobiles.</t>
+          <t>Oct rent, Oct mobiles. (Complete AV labour was released and paid 8 Oct, so nothing held now.)</t>
         </is>
       </c>
     </row>
@@ -3280,14 +3280,14 @@
     <row r="69" ht="15.75" customHeight="1" s="109">
       <c r="A69" s="110" t="inlineStr">
         <is>
-          <t>1. Aware Super $225,887 (INV-10596) is the big one - still not paid at 12 Oct and now expected 9 Nov, after this forecast. Complete AV materials $133,246 went out 29 Sep. If Aware slip again the held labour stays held and we watch the cheque account. Build-up on the Complete AV tab.</t>
+          <t>1. Aware Super $225,887 (INV-10596) is the big one - still not paid at 12 Oct and now expected 9 Nov, after this forecast. The whole Complete AV bill ($178,119) is now paid ahead of it (materials 29 Sep, labour 8 Oct), so we watch the cheque account until Aware pay. Build-up on the Complete AV tab.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15.75" customHeight="1" s="109">
       <c r="A70" s="110" t="inlineStr">
         <is>
-          <t>2. Complete AV labour and programming ($41,956 inc GST) is held until Aware sign off and we get the handover docs - agreed 28 Sep. Jordan thinks they may push for programming or sub-trade costs. If we agree to any, add them on the Payables tab.</t>
+          <t>2. Complete AV labour and programming ($39,033 inc GST) was released and paid 8 Oct, so INV41565 is fully paid. The $5,334 balance of the quote is still to be invoiced (claim 3). Jordan thinks they may push for programming or sub-trade costs - if we agree to any, add them on the Payables tab.</t>
         </is>
       </c>
     </row>
@@ -7924,23 +7924,23 @@
     </row>
     <row r="14">
       <c r="A14" s="176" t="str">
-        <f>A34</f>
-        <v>Posh Services (Ambius)</v>
+        <f>A21</f>
+        <v>Complete AV Solutions</v>
       </c>
       <c r="B14" s="177" t="str">
-        <f>B34</f>
-        <v>INV21736844 - indoor plants Sep</v>
+        <f>B21</f>
+        <v>INV41565 - Aware seminar room: LABOUR &amp; PROGRAMMING portion - released</v>
       </c>
       <c r="C14" s="178">
-        <f>C34</f>
-        <v>46304</v>
+        <f>C21</f>
+        <v>46291</v>
       </c>
       <c r="D14" s="179">
-        <f>D34</f>
-        <v>245</v>
+        <f>D21</f>
+        <v>39033.020000000004</v>
       </c>
       <c r="E14" s="176" t="str">
-        <f>E34</f>
+        <f>E21</f>
         <v>EFT</v>
       </c>
       <c r="F14" s="180" t="inlineStr">
@@ -7949,14 +7949,14 @@
         </is>
       </c>
       <c r="G14" s="181">
-        <f>G34</f>
+        <f>G21</f>
         <v>46303</v>
       </c>
       <c r="H14" s="182" t="n"/>
       <c r="I14" s="182" t="n"/>
       <c r="J14" s="175" t="inlineStr">
         <is>
-          <t>Posh plants - paid</t>
+          <t>Complete AV labour and programming - hold released, paid</t>
         </is>
       </c>
     </row>
@@ -7970,7 +7970,7 @@
       <c r="C15" s="16" t="n"/>
       <c r="D15" s="142">
         <f>SUM(D6:D14)</f>
-        <v>76418.96999999999</v>
+        <v>115206.98999999999</v>
       </c>
       <c r="E15" s="16" t="n"/>
       <c r="F15" s="16" t="n"/>
@@ -8137,53 +8137,53 @@
       </c>
       <c r="J20" s="175" t="inlineStr">
         <is>
-          <t>PAID 29 Sep (Xero shows the whole bill as paid 8 Oct - see note on the hold).</t>
+          <t>PAID 29 Sep</t>
         </is>
       </c>
     </row>
     <row r="21" ht="72" customHeight="1" s="109">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="170" t="inlineStr">
         <is>
           <t>Complete AV Solutions</t>
         </is>
       </c>
-      <c r="B21" s="110" t="inlineStr">
-        <is>
-          <t>INV41565 - Aware seminar room: LABOUR &amp; PROGRAMMING portion - HELD</t>
-        </is>
-      </c>
-      <c r="C21" s="137" t="n">
+      <c r="B21" s="183" t="inlineStr">
+        <is>
+          <t>INV41565 - Aware seminar room: LABOUR &amp; PROGRAMMING portion - released</t>
+        </is>
+      </c>
+      <c r="C21" s="171" t="n">
         <v>46291</v>
       </c>
-      <c r="D21" s="148">
+      <c r="D21" s="179">
         <f>'Complete AV'!L19-'Complete AV'!L22</f>
         <v>39033.020000000004</v>
       </c>
-      <c r="E21" s="33" t="inlineStr">
+      <c r="E21" s="173" t="inlineStr">
         <is>
           <t>EFT</t>
         </is>
       </c>
-      <c r="F21" s="33" t="inlineStr">
+      <c r="F21" s="173" t="inlineStr">
         <is>
           <t>Equipment purchases</t>
         </is>
       </c>
-      <c r="G21" s="141" t="n">
-        <v>46356</v>
-      </c>
-      <c r="H21" s="18" t="str">
+      <c r="G21" s="171" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H21" s="170">
         <f>IF(G21&lt;Assumptions!$B$5,"Before",IF(G21&gt;Assumptions!$C$48,"After",INT((G21-Assumptions!$B$5)/7)+1))</f>
-        <v>After</v>
-      </c>
-      <c r="I21" s="18" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="I21" s="170" t="inlineStr">
         <is>
           <t>Xero bill</t>
         </is>
       </c>
-      <c r="J21" s="115" t="inlineStr">
-        <is>
-          <t>HELD - agreed 28 Sep, released on Aware sign off and handover docs. Xero shows INV41565 fully paid on 8 Oct ($178,119.25) - if the $44,873 did go out, it needs to go into week 2 actuals.</t>
+      <c r="J21" s="175" t="inlineStr">
+        <is>
+          <t>PAID 8 Oct - the hold was released last week. Whole of INV41565 ($178,119.25) is now paid, matches Xero.</t>
         </is>
       </c>
     </row>
@@ -10571,12 +10571,12 @@
     <row r="80" s="109">
       <c r="A80" s="29" t="inlineStr">
         <is>
-          <t>Non-card bills dated past the forecast (Complete AV labour hold, Oct rent, Oct mobiles)</t>
+          <t>Non-card bills dated past the forecast (Oct rent, Oct mobiles)</t>
         </is>
       </c>
       <c r="D80" s="143">
         <f>SUMIFS(D19:D75,E19:E75,"&lt;&gt;Card",G19:G75,"&gt;"&amp;Assumptions!$C$48)</f>
-        <v>69117.8</v>
+        <v>30084.780000000002</v>
       </c>
     </row>
   </sheetData>
@@ -10619,14 +10619,14 @@
     <row r="1" ht="18" customHeight="1" s="109">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Complete AV Solutions - INV41565 - what we're paying and what's held</t>
+          <t>Complete AV Solutions - INV41565 - what we paid and when</t>
         </is>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" s="109">
       <c r="A2" s="115" t="inlineStr">
         <is>
-          <t>Aware Super seminar room audio upgrade (Q-12140v1, PO-00016902). Bill total $178,119.25 inc GST, dated 1 Sep, due 26 Sep. Agreed 28 Sep (Graham / Jordan): pay the materials now, hold labour and programming until Aware sign off and we get the handover docs. Line items are straight off the bill in Xero.</t>
+          <t>Aware Super seminar room audio upgrade (Q-12140v1, PO-00016902). Bill total $178,119.25 inc GST, dated 1 Sep, due 26 Sep. Agreed 28 Sep (Graham / Jordan): pay the materials now, hold labour and programming until Aware sign off and we get the handover docs. Line items are straight off the bill in Xero. Update 12 Oct: the labour and programming that was held ($39,033.02) was released and paid Thu 8 Oct, so the whole bill is now paid.</t>
         </is>
       </c>
       <c r="G2" s="116" t="inlineStr">
@@ -11577,7 +11577,7 @@
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>HELD - labour and programming (until Aware sign off + handover docs)</t>
+          <t>LABOUR AND PROGRAMMING - was held, released and PAID Thu 8 Oct</t>
         </is>
       </c>
       <c r="B48" s="114" t="n"/>

</xml_diff>

<commit_message>
Cash flow: 6 Oct pay run and 7 Oct super/payroll tax into week 1 from Xero bank, Tuesday pay dates restored
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141HuBtr9dZXPeYR1jN9h28
</commit_message>
<xml_diff>
--- a/cashflow/CTS Cash Flow Forecast - 12102026.xlsx
+++ b/cashflow/CTS Cash Flow Forecast - 12102026.xlsx
@@ -1107,7 +1107,7 @@
       <c r="N8" s="12" t="n"/>
       <c r="O8" s="76" t="inlineStr">
         <is>
-          <t>Week 1 is done and ties to CommBiz. Week 2 actuals are in to Mon 12 Oct only - flag stays 0 until the week closes Wed 14 Oct and the bank balance is keyed.</t>
+          <t>Week 1 is done and reconciles to Xero (flag 1). Week 2 actuals are in to Mon 12 Oct only - flag stays 0 until the week closes Wed 14 Oct and the bank balance is keyed.</t>
         </is>
       </c>
     </row>
@@ -1127,35 +1127,35 @@
       </c>
       <c r="D10" s="119">
         <f>IF(C$8=1,C59,B58)</f>
-        <v>358696.23</v>
+        <v>261747.39999999997</v>
       </c>
       <c r="E10" s="119">
         <f>D10</f>
-        <v>358696.23</v>
+        <v>261747.39999999997</v>
       </c>
       <c r="F10" s="119">
         <f>IF(E$8=1,E59,D58)</f>
-        <v>261282.50999999998</v>
+        <v>263901.67999999993</v>
       </c>
       <c r="G10" s="119">
         <f>F10</f>
-        <v>261282.50999999998</v>
+        <v>263901.67999999993</v>
       </c>
       <c r="H10" s="119">
         <f>IF(G$8=1,G59,F58)</f>
-        <v>495886.79666666663</v>
+        <v>498505.9666666666</v>
       </c>
       <c r="I10" s="119">
         <f>H10</f>
-        <v>495886.79666666663</v>
+        <v>498505.9666666666</v>
       </c>
       <c r="J10" s="119">
         <f>IF(I$8=1,I59,H58)</f>
-        <v>230920.72933333332</v>
+        <v>333107.8993333333</v>
       </c>
       <c r="K10" s="119">
         <f>J10</f>
-        <v>230920.72933333332</v>
+        <v>333107.8993333333</v>
       </c>
       <c r="L10" s="119">
         <f>B10</f>
@@ -1200,8 +1200,8 @@
         <v>134590.91999999998</v>
       </c>
       <c r="C13" s="121">
-        <f>41925.4+6172.39+58024.76+1975.51+1092.3+13046.62+4352.45+13156</f>
-        <v>139745.43</v>
+        <f>41925.4+6172.39+58024.76+1975.51+1092.3+13046.62+4352.45+13156+9350+93.5+627+8043.2</f>
+        <v>157859.13</v>
       </c>
       <c r="D13" s="120">
         <f>SUMIFS(Receivables!$F$5:$F$65,Receivables!$H$5:$H$65,"&gt;="&amp;Assumptions!$B$45,Receivables!$H$5:$H$65,"&lt;="&amp;Assumptions!$C$45)</f>
@@ -1232,15 +1232,15 @@
       </c>
       <c r="M13" s="120">
         <f>SUM(C13,E13,G13,I13,K13)</f>
-        <v>282947.7</v>
+        <v>301061.4</v>
       </c>
       <c r="N13" s="120">
         <f>(C13-B13)*C$8+(E13-D13)*E$8+(G13-F13)*G$8+(I13-H13)*I$8+(K13-J13)*K$8</f>
-        <v>5154.510000000009</v>
+        <v>23268.21000000002</v>
       </c>
       <c r="O13" s="108" t="inlineStr">
         <is>
-          <t>Week 2 to 12 Oct: Deloitte $112,683.22 and $18,891.66, CEO Institute $9,086.39, ASX $1,661, Dimensional $506, Ricoh $374 (Xero). Nothing from Aware yet.</t>
+          <t>Week 1 now includes 6-7 Oct: PwC $9,350, CBA Melb $93.50, APA $627, CBA Bris $8,043.20. Week 2 to 12 Oct: Deloitte $112,683.22 and $18,891.66, CEO Institute $9,086.39, ASX $1,661, Dimensional $506, Ricoh $374. Nothing from Aware yet.</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="C15" s="122">
         <f>C13+C14</f>
-        <v>140175.6</v>
+        <v>158289.30000000002</v>
       </c>
       <c r="D15" s="122">
         <f>D13+D14</f>
@@ -1349,11 +1349,11 @@
       </c>
       <c r="M15" s="122">
         <f>M13+M14</f>
-        <v>283377.87</v>
+        <v>301491.57</v>
       </c>
       <c r="N15" s="122">
         <f>N13+N14</f>
-        <v>5584.680000000009</v>
+        <v>23698.38000000002</v>
       </c>
       <c r="O15" s="16" t="n"/>
     </row>
@@ -1393,44 +1393,49 @@
       </c>
       <c r="B19" s="120">
         <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$44,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$44)</f>
-        <v>0</v>
-      </c>
-      <c r="C19" s="121" t="n"/>
+        <v>85248</v>
+      </c>
+      <c r="C19" s="121">
+        <f>71172.55+9443.5-880</f>
+        <v>79736.05</v>
+      </c>
       <c r="D19" s="120">
         <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$45,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$45)</f>
-        <v>85248</v>
-      </c>
-      <c r="E19" s="121" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="E19" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="F19" s="120">
         <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$46,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$46)</f>
-        <v>0</v>
+        <v>85248</v>
       </c>
       <c r="G19" s="121" t="n"/>
       <c r="H19" s="120">
         <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$47,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$47)</f>
-        <v>85248</v>
+        <v>0</v>
       </c>
       <c r="I19" s="121" t="n"/>
       <c r="J19" s="120">
         <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$48,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$48)</f>
-        <v>0</v>
+        <v>85248</v>
       </c>
       <c r="K19" s="121" t="n"/>
       <c r="L19" s="120">
         <f>SUM(B19,D19,F19,H19,J19)</f>
-        <v>170496</v>
+        <v>255744</v>
       </c>
       <c r="M19" s="120">
         <f>SUM(C19,E19,G19,I19,K19)</f>
-        <v>0</v>
+        <v>79736.05</v>
       </c>
       <c r="N19" s="120">
         <f>(C19-B19)*C$8+(E19-D19)*E$8+(G19-F19)*G$8+(I19-H19)*I$8+(K19-J19)*K$8</f>
-        <v>0</v>
+        <v>-5511.949999999997</v>
       </c>
       <c r="O19" s="108" t="inlineStr">
         <is>
-          <t>Payroll tab - gross x net %. Fortnight is Sat to Fri and the money goes out the Tuesday after: Tue 13 Oct (week 2) and Tue 27 Oct (week 4). The next one is Tue 10 Nov, after this forecast.</t>
+          <t>Payroll tab - gross x net %. Fortnight is Sat to Fri and the money goes out the Tuesday after: Tue 6 Oct (week 1), Tue 20 Oct (week 3) and Tue 3 Nov (week 5). 6 Oct actual is from the Xero bank movement - swap in the ABA figure.</t>
         </is>
       </c>
     </row>
@@ -1442,40 +1447,44 @@
       </c>
       <c r="B20" s="120">
         <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$44,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$44)</f>
-        <v>0</v>
-      </c>
-      <c r="C20" s="121" t="n"/>
+        <v>13320</v>
+      </c>
+      <c r="C20" s="121" t="n">
+        <v>13083.54</v>
+      </c>
       <c r="D20" s="120">
         <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$45,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$45)</f>
-        <v>13320</v>
-      </c>
-      <c r="E20" s="121" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="E20" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="F20" s="120">
         <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$46,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$46)</f>
-        <v>0</v>
+        <v>13320</v>
       </c>
       <c r="G20" s="121" t="n"/>
       <c r="H20" s="120">
         <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$47,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$47)</f>
-        <v>13320</v>
+        <v>0</v>
       </c>
       <c r="I20" s="121" t="n"/>
       <c r="J20" s="120">
         <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$48,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$48)</f>
-        <v>0</v>
+        <v>13320</v>
       </c>
       <c r="K20" s="121" t="n"/>
       <c r="L20" s="120">
         <f>SUM(B20,D20,F20,H20,J20)</f>
-        <v>26640</v>
+        <v>39960</v>
       </c>
       <c r="M20" s="120">
         <f>SUM(C20,E20,G20,I20,K20)</f>
-        <v>0</v>
+        <v>13083.54</v>
       </c>
       <c r="N20" s="120">
         <f>(C20-B20)*C$8+(E20-D20)*E$8+(G20-F20)*G$8+(I20-H20)*I$8+(K20-J20)*K$8</f>
-        <v>0</v>
+        <v>-236.45999999999913</v>
       </c>
       <c r="O20" s="108" t="inlineStr">
         <is>
@@ -1544,7 +1553,9 @@
         <f>IF(AND(Assumptions!$B$19&gt;=Assumptions!$B$44,Assumptions!$B$19&lt;=Assumptions!$C$44),Assumptions!$B$17+Assumptions!$B$18,0)</f>
         <v>8995</v>
       </c>
-      <c r="C22" s="121" t="n"/>
+      <c r="C22" s="121" t="n">
+        <v>8602.75</v>
+      </c>
       <c r="D22" s="120">
         <f>IF(AND(Assumptions!$B$19&gt;=Assumptions!$B$45,Assumptions!$B$19&lt;=Assumptions!$C$45),Assumptions!$B$17+Assumptions!$B$18,0)</f>
         <v>0</v>
@@ -1573,15 +1584,15 @@
       </c>
       <c r="M22" s="120">
         <f>SUM(C22,E22,G22,I22,K22)</f>
-        <v>0</v>
+        <v>8602.75</v>
       </c>
       <c r="N22" s="120">
         <f>(C22-B22)*C$8+(E22-D22)*E$8+(G22-F22)*G$8+(I22-H22)*I$8+(K22-J22)*K$8</f>
-        <v>-8995</v>
+        <v>-392.25</v>
       </c>
       <c r="O22" s="108" t="inlineStr">
         <is>
-          <t>Sep wages, due 7 Oct. Aug numbers used until the Sep return is lodged ($6,295 NSW + $2,700 other states).</t>
+          <t>Sep wages, due 7 Oct. Paid Wed 7 Oct - $8,602.75 per Xero. Aug numbers were used for the forecast ($6,295 NSW + $2,700 other).</t>
         </is>
       </c>
     </row>
@@ -1593,32 +1604,34 @@
       </c>
       <c r="B23" s="120">
         <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$44,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$44)</f>
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="C23" s="121" t="n"/>
       <c r="D23" s="120">
         <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$45,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$45)</f>
-        <v>1000</v>
-      </c>
-      <c r="E23" s="121" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="E23" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="F23" s="120">
         <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$46,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$46)</f>
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="G23" s="121" t="n"/>
       <c r="H23" s="120">
         <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$47,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$47)</f>
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I23" s="121" t="n"/>
       <c r="J23" s="120">
         <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$48,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$48)</f>
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="K23" s="121" t="n"/>
       <c r="L23" s="120">
         <f>SUM(B23,D23,F23,H23,J23)</f>
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="M23" s="120">
         <f>SUM(C23,E23,G23,I23,K23)</f>
@@ -1626,11 +1639,11 @@
       </c>
       <c r="N23" s="120">
         <f>(C23-B23)*C$8+(E23-D23)*E$8+(G23-F23)*G$8+(I23-H23)*I$8+(K23-J23)*K$8</f>
-        <v>0</v>
+        <v>-1000</v>
       </c>
       <c r="O23" s="108" t="inlineStr">
         <is>
-          <t>Placeholder. Week 2 actual gets filled on pay day Tue 13 Oct.</t>
+          <t>Placeholder. Expense claims go out with the ABA, so the 6 Oct actual net pay already has them in it.</t>
         </is>
       </c>
     </row>
@@ -1642,15 +1655,15 @@
       </c>
       <c r="B24" s="123">
         <f>B19+B20+B21+B22+B23</f>
-        <v>8995</v>
+        <v>108563</v>
       </c>
       <c r="C24" s="123">
         <f>C19+C20+C21+C22+C23</f>
-        <v>0</v>
+        <v>101422.34</v>
       </c>
       <c r="D24" s="123">
         <f>D19+D20+D21+D22+D23</f>
-        <v>99568</v>
+        <v>0</v>
       </c>
       <c r="E24" s="123">
         <f>E19+E20+E21+E22+E23</f>
@@ -1658,7 +1671,7 @@
       </c>
       <c r="F24" s="123">
         <f>F19+F20+F21+F22+F23</f>
-        <v>0</v>
+        <v>99568</v>
       </c>
       <c r="G24" s="123">
         <f>G19+G20+G21+G22+G23</f>
@@ -1666,7 +1679,7 @@
       </c>
       <c r="H24" s="123">
         <f>H19+H20+H21+H22+H23</f>
-        <v>99568</v>
+        <v>0</v>
       </c>
       <c r="I24" s="123">
         <f>I19+I20+I21+I22+I23</f>
@@ -1674,7 +1687,7 @@
       </c>
       <c r="J24" s="123">
         <f>J19+J20+J21+J22+J23</f>
-        <v>0</v>
+        <v>99568</v>
       </c>
       <c r="K24" s="123">
         <f>K19+K20+K21+K22+K23</f>
@@ -1682,15 +1695,15 @@
       </c>
       <c r="L24" s="123">
         <f>L19+L20+L21+L22+L23</f>
-        <v>208131</v>
+        <v>307699</v>
       </c>
       <c r="M24" s="123">
         <f>M19+M20+M21+M22+M23</f>
-        <v>0</v>
+        <v>101422.34</v>
       </c>
       <c r="N24" s="123">
         <f>N19+N20+N21+N22+N23</f>
-        <v>-8995</v>
+        <v>-7140.659999999996</v>
       </c>
       <c r="O24" s="12" t="n"/>
     </row>
@@ -2193,7 +2206,9 @@
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$44,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$44,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Professional fees")+Assumptions!$B$33/5</f>
         <v>1680</v>
       </c>
-      <c r="C38" s="121" t="n"/>
+      <c r="C38" s="121" t="n">
+        <v>880</v>
+      </c>
       <c r="D38" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Professional fees")+Assumptions!$B$33/5</f>
         <v>1680</v>
@@ -2222,11 +2237,11 @@
       </c>
       <c r="M38" s="120">
         <f>SUM(C38,E38,G38,I38,K38)</f>
-        <v>0</v>
+        <v>880</v>
       </c>
       <c r="N38" s="120">
         <f>(C38-B38)*C$8+(E38-D38)*E$8+(G38-F38)*G$8+(I38-H38)*I$8+(K38-J38)*K$8</f>
-        <v>-1680</v>
+        <v>-800</v>
       </c>
       <c r="O38" s="108" t="inlineStr">
         <is>
@@ -2606,7 +2621,9 @@
         <f>Assumptions!$B$37/5</f>
         <v>5000</v>
       </c>
-      <c r="C46" s="121" t="n"/>
+      <c r="C46" s="121" t="n">
+        <v>10000</v>
+      </c>
       <c r="D46" s="120">
         <f>Assumptions!$B$37/5</f>
         <v>5000</v>
@@ -2635,15 +2652,15 @@
       </c>
       <c r="M46" s="120">
         <f>SUM(C46,E46,G46,I46,K46)</f>
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="N46" s="120">
         <f>(C46-B46)*C$8+(E46-D46)*E$8+(G46-F46)*G$8+(I46-H46)*I$8+(K46-J46)*K$8</f>
-        <v>-5000</v>
+        <v>5000</v>
       </c>
       <c r="O46" s="108" t="inlineStr">
         <is>
-          <t>~$25k a month transferred to the PL and DL cards. Covers every Card row on the Payables tab (subscriptions, travel, electricity, Seek, Goget, EH).</t>
+          <t>~$25k a month transferred to the PL and DL cards. Covers every Card row on the Payables tab (subscriptions, travel, electricity, Seek, Goget, EH). Week 1 actual: $10,000 moved to the PL card 7 Oct.</t>
         </is>
       </c>
     </row>
@@ -2733,7 +2750,7 @@
       </c>
       <c r="C49" s="123">
         <f>C35+C36+C37+C38+C39+C40+C41+C42+C43+C44+C45+C46+C47+C48</f>
-        <v>77548.14</v>
+        <v>88428.14</v>
       </c>
       <c r="D49" s="123">
         <f>D35+D36+D37+D38+D39+D40+D41+D42+D43+D44+D45+D46+D47</f>
@@ -2773,11 +2790,11 @@
       </c>
       <c r="M49" s="123">
         <f>M35+M36+M37+M38+M39+M40+M41+M42+M43+M44+M45+M46+M47</f>
-        <v>1430.71</v>
+        <v>12310.71</v>
       </c>
       <c r="N49" s="123">
         <f>N35+N36+N37+N38+N39+N40+N41+N42+N43+N44+N45+N46+N47</f>
-        <v>-14870</v>
+        <v>-3990</v>
       </c>
       <c r="O49" s="12" t="n"/>
     </row>
@@ -2906,15 +2923,15 @@
       </c>
       <c r="B55" s="122">
         <f>B24+B32+B49+B53</f>
-        <v>213633.83</v>
+        <v>313201.82999999996</v>
       </c>
       <c r="C55" s="122">
         <f>C24+C32+C49+C53</f>
-        <v>216634.37</v>
+        <v>328936.71</v>
       </c>
       <c r="D55" s="122">
         <f>D24+D32+D49+D53</f>
-        <v>240109.99</v>
+        <v>140541.99</v>
       </c>
       <c r="E55" s="122">
         <f>E24+E32+E49+E53</f>
@@ -2922,7 +2939,7 @@
       </c>
       <c r="F55" s="122">
         <f>F24+F32+F49+F66</f>
-        <v>60002.060000000005</v>
+        <v>159570.06</v>
       </c>
       <c r="G55" s="122">
         <f>G24+G32+G49+G53</f>
@@ -2930,7 +2947,7 @@
       </c>
       <c r="H55" s="122">
         <f>H24+H32+H49+H53</f>
-        <v>277592.534</v>
+        <v>178024.53399999999</v>
       </c>
       <c r="I55" s="122">
         <f>I24+I32+I49+I53</f>
@@ -2938,7 +2955,7 @@
       </c>
       <c r="J55" s="122">
         <f>J24+J32+J49+J53</f>
-        <v>52650.92</v>
+        <v>152218.92</v>
       </c>
       <c r="K55" s="122">
         <f>K24+K32+K49+K53</f>
@@ -2946,15 +2963,15 @@
       </c>
       <c r="L55" s="122">
         <f>L24+L32+L49+L53</f>
-        <v>843989.3339999999</v>
+        <v>943557.3339999999</v>
       </c>
       <c r="M55" s="122">
         <f>M24+M32+M49+M53</f>
-        <v>258393.89999999997</v>
+        <v>370696.24</v>
       </c>
       <c r="N55" s="122">
         <f>N24+N32+N49+N53</f>
-        <v>-74301.99999999999</v>
+        <v>-61567.65999999998</v>
       </c>
       <c r="O55" s="16" t="n"/>
     </row>
@@ -2966,15 +2983,15 @@
       </c>
       <c r="B57" s="122">
         <f>B15-B55</f>
-        <v>-79042.91</v>
+        <v>-178610.90999999997</v>
       </c>
       <c r="C57" s="122">
         <f>C15-C55</f>
-        <v>-76458.76999999999</v>
+        <v>-170647.41</v>
       </c>
       <c r="D57" s="122">
         <f>D15-D55</f>
-        <v>-97413.72</v>
+        <v>2154.279999999999</v>
       </c>
       <c r="E57" s="122">
         <f>E15-E55</f>
@@ -2990,7 +3007,7 @@
       </c>
       <c r="H57" s="122">
         <f>H15-H55</f>
-        <v>-264966.0673333333</v>
+        <v>-165398.0673333333</v>
       </c>
       <c r="I57" s="122">
         <f>I15-I55</f>
@@ -2998,7 +3015,7 @@
       </c>
       <c r="J57" s="122">
         <f>J15-J55</f>
-        <v>39819.21666666666</v>
+        <v>-59748.783333333355</v>
       </c>
       <c r="K57" s="122">
         <f>K15-K55</f>
@@ -3006,15 +3023,15 @@
       </c>
       <c r="L57" s="122">
         <f>L15-L55</f>
-        <v>-227001.25400000007</v>
+        <v>-326569.2540000001</v>
       </c>
       <c r="M57" s="122">
         <f>M15-M55</f>
-        <v>24983.97000000003</v>
+        <v>-69204.66999999998</v>
       </c>
       <c r="N57" s="122">
         <f>N15-N55</f>
-        <v>79886.68</v>
+        <v>85266.04000000001</v>
       </c>
       <c r="O57" s="16" t="n"/>
     </row>
@@ -3026,15 +3043,15 @@
       </c>
       <c r="B58" s="125">
         <f>B10+B57</f>
-        <v>356112.08999999997</v>
+        <v>256544.09000000003</v>
       </c>
       <c r="C58" s="125">
         <f>C10+C57</f>
-        <v>358696.23</v>
+        <v>264507.58999999997</v>
       </c>
       <c r="D58" s="125">
         <f>D10+D57</f>
-        <v>261282.50999999998</v>
+        <v>263901.67999999993</v>
       </c>
       <c r="E58" s="125" t="str">
         <f>IF(E$8=1,E10+E57,"")</f>
@@ -3042,7 +3059,7 @@
       </c>
       <c r="F58" s="125">
         <f>F10+F57</f>
-        <v>495886.79666666663</v>
+        <v>498505.9666666666</v>
       </c>
       <c r="G58" s="125" t="str">
         <f>IF(G$8=1,G10+G57,"")</f>
@@ -3050,7 +3067,7 @@
       </c>
       <c r="H58" s="125">
         <f>H10+H57</f>
-        <v>230920.72933333332</v>
+        <v>333107.8993333333</v>
       </c>
       <c r="I58" s="125" t="str">
         <f>IF(I$8=1,I10+I57,"")</f>
@@ -3058,7 +3075,7 @@
       </c>
       <c r="J58" s="125">
         <f>J10+J57</f>
-        <v>270739.946</v>
+        <v>273359.1159999999</v>
       </c>
       <c r="K58" s="125" t="str">
         <f>IF(K$8=1,K10+K57,"")</f>
@@ -3066,11 +3083,11 @@
       </c>
       <c r="L58" s="125">
         <f>J58</f>
-        <v>270739.946</v>
+        <v>273359.1159999999</v>
       </c>
       <c r="M58" s="125">
         <f>IF(K$8=1,K58,IF(I$8=1,I58,IF(G$8=1,G58,IF(E$8=1,E58,IF(C$8=1,C58,"")))))</f>
-        <v>358696.23</v>
+        <v>264507.58999999997</v>
       </c>
       <c r="N58" s="26" t="n"/>
       <c r="O58" s="78" t="inlineStr">
@@ -3087,8 +3104,8 @@
       </c>
       <c r="B59" s="10" t="n"/>
       <c r="C59" s="121">
-        <f>88266.06+270430.17</f>
-        <v>358696.23</v>
+        <f>358696.23-86948.83-10000</f>
+        <v>261747.39999999997</v>
       </c>
       <c r="D59" s="10" t="n"/>
       <c r="E59" s="121" t="n"/>
@@ -3103,7 +3120,7 @@
       <c r="N59" s="12" t="n"/>
       <c r="O59" s="79" t="inlineStr">
         <is>
-          <t>Type the real closing balance (cheque + savings) in at the end of each week. Week 2 - key it Wed 14 Oct, then set the flag to 1.</t>
+          <t>Type the real closing balance (cheque + savings) in at the end of each week. Week 1 is worked back from Xero: $358,696.23 at Mon 5 Oct, less the $86,948.83 Xero cash drop over 6-7 Oct and the $10k card transfer - replace with the CommBiz 7 Oct figure. Week 2 - key it Wed 14 Oct, then set the flag to 1.</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3133,7 @@
       <c r="B60" s="10" t="n"/>
       <c r="C60" s="126">
         <f>C58-C59</f>
-        <v>0</v>
+        <v>2760.1900000000023</v>
       </c>
       <c r="D60" s="10" t="n"/>
       <c r="E60" s="126" t="str">
@@ -3143,7 +3160,7 @@
       <c r="N60" s="12" t="n"/>
       <c r="O60" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Should be nil once everything's in. this is a sense check </t>
+          <t>Should be nil once everything's in. Week 1 is about $2.8k unexplained - small card / bank items on 6-7 Oct that aren't on a bill. Clears when the real 7 Oct balance goes in.</t>
         </is>
       </c>
     </row>
@@ -3176,23 +3193,23 @@
       </c>
       <c r="B63" s="120">
         <f>B19+B20+B23</f>
-        <v>0</v>
+        <v>99568</v>
       </c>
       <c r="D63" s="120">
         <f>D19+D20+D23</f>
-        <v>99568</v>
+        <v>0</v>
       </c>
       <c r="F63" s="120">
         <f>F19+F20+F23</f>
-        <v>0</v>
+        <v>99568</v>
       </c>
       <c r="H63" s="120">
         <f>H19+H20+H23</f>
-        <v>99568</v>
+        <v>0</v>
       </c>
       <c r="J63" s="120">
         <f>J19+J20+J23</f>
-        <v>0</v>
+        <v>99568</v>
       </c>
       <c r="O63" s="108" t="n"/>
     </row>
@@ -3204,23 +3221,23 @@
       </c>
       <c r="B64" s="127">
         <f>IF(Payroll!$I$5=0,0,B58/(Payroll!$I$5/2))</f>
-        <v>7.153143379399003</v>
+        <v>5.153143379399004</v>
       </c>
       <c r="D64" s="127">
         <f>IF(Payroll!$I$5=0,0,D58/(Payroll!$I$5/2))</f>
-        <v>5.248322955166318</v>
+        <v>5.300933633295837</v>
       </c>
       <c r="F64" s="127">
         <f>IF(Payroll!$I$5=0,0,F58/(Payroll!$I$5/2))</f>
-        <v>9.960766444373023</v>
+        <v>10.013377122502543</v>
       </c>
       <c r="H64" s="127">
         <f>IF(Payroll!$I$5=0,0,H58/(Payroll!$I$5/2))</f>
-        <v>4.638452702340778</v>
+        <v>6.691063380470298</v>
       </c>
       <c r="J64" s="127">
         <f>IF(Payroll!$I$5=0,0,J58/(Payroll!$I$5/2))</f>
-        <v>5.438292342921421</v>
+        <v>5.490903021050938</v>
       </c>
       <c r="O64" s="108" t="n"/>
     </row>
@@ -3377,7 +3394,7 @@
       </c>
       <c r="C5" s="115" t="inlineStr">
         <is>
-          <t>Mon 28 Sep. Week 1 runs through to Wed 7 Oct so it picks up payroll tax on the 7th, then it's weekly from there (Thu to Wed). Week table is at the bottom of this tab.</t>
+          <t>Mon 28 Sep. Week 1 runs through to Wed 7 Oct so it picks up the 6 Oct pay run and payroll tax on the 7th, then it's weekly from there (Thu to Wed). Week table is at the bottom of this tab.</t>
         </is>
       </c>
     </row>
@@ -3500,45 +3517,45 @@
     <row r="14" ht="24" customHeight="1" s="109">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>Pay date - run 1 (fortnight Sat 26 Sep to Fri 9 Oct)</t>
+          <t>Pay date - run 1 (fortnight Sat 19 Sep to Fri 2 Oct)</t>
         </is>
       </c>
       <c r="B14" s="128" t="n">
-        <v>46308</v>
+        <v>46301</v>
       </c>
       <c r="C14" s="115" t="inlineStr">
         <is>
-          <t>Fortnight is Sat 26 Sep to Fri 9 Oct. Processed Mon 12 Oct, out of the bank Tue 13 Oct (week 2). Xero has the pay run journal dated 8-9 Oct for $101,246 gross - that is the journal date, the money goes on the Tuesday. Super direct debits the same week - payday super since 1 Jul 26.</t>
+          <t>Fortnight Sat 19 Sep to Fri 2 Oct, out of the bank Tue 6 Oct (week 1). Xero bank shows about $79.7k leaving on the 6th and super + payroll tax on the 7th - the pay run journal is just dated 8-9 Oct. Super direct debits the day after - payday super since 1 Jul 26.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t>Pay date - run 2 (fortnight Sat 10 Oct to Fri 23 Oct)</t>
+          <t>Pay date - run 2 (fortnight Sat 3 Oct to Fri 16 Oct)</t>
         </is>
       </c>
       <c r="B15" s="128" t="n">
-        <v>46322</v>
+        <v>46315</v>
       </c>
       <c r="C15" s="115" t="inlineStr">
         <is>
-          <t>Tue 27 Oct (week 4).</t>
+          <t>Tue 20 Oct (week 3).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="18" t="inlineStr">
         <is>
-          <t>Pay date - run 3 (fortnight Sat 24 Oct to Fri 6 Nov)</t>
+          <t>Pay date - run 3 (fortnight Sat 17 Oct to Fri 30 Oct)</t>
         </is>
       </c>
       <c r="B16" s="128" t="n">
-        <v>46336</v>
+        <v>46329</v>
       </c>
       <c r="C16" s="115" t="inlineStr">
         <is>
-          <t>Tue 10 Nov - after week 5 (ends Wed 4 Nov), so it does not hit this forecast. Only two pay runs land in October now.</t>
+          <t>Tue 3 Nov (week 5).</t>
         </is>
       </c>
     </row>
@@ -4067,15 +4084,15 @@
     <row r="5" ht="48" customHeight="1" s="109">
       <c r="A5" s="18" t="inlineStr">
         <is>
-          <t>Run 1 - Sat 26 Sep to Fri 9 Oct</t>
+          <t>Run 1 - Sat 19 Sep to Fri 2 Oct</t>
         </is>
       </c>
       <c r="B5" s="128" t="n">
-        <v>46304</v>
+        <v>46297</v>
       </c>
       <c r="C5" s="135">
         <f>Assumptions!$B$14</f>
-        <v>46308</v>
+        <v>46301</v>
       </c>
       <c r="D5" s="136">
         <f>Assumptions!$B$9</f>
@@ -4103,22 +4120,22 @@
       </c>
       <c r="J5" s="115" t="inlineStr">
         <is>
-          <t>Timesheets close Fri 9 Oct, processed Mon 12 Oct - approvals, reconcile, finalise with GC, ABA into CommBiz, payroll email to DL. Move the funds from savings Monday. Out of the bank Tue 13 Oct. Xero journal is dated 8-9 Oct ($101,246 gross, $13,084 super).</t>
+          <t>Timesheets closed Fri 2 Oct, Mon 5 Oct was a PH, out of the bank Tue 6 Oct - Xero bank movement says about $79.7k net (78.8% of the $101,246 gross). Super $13,084 and payroll tax $8,603 went Wed 7 Oct. Journal in Xero is dated 8-9 Oct.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" s="109">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Run 2 - Sat 10 Oct to Fri 23 Oct</t>
+          <t>Run 2 - Sat 3 Oct to Fri 16 Oct</t>
         </is>
       </c>
       <c r="B6" s="128" t="n">
-        <v>46318</v>
+        <v>46311</v>
       </c>
       <c r="C6" s="135">
         <f>Assumptions!$B$15</f>
-        <v>46322</v>
+        <v>46315</v>
       </c>
       <c r="D6" s="136">
         <f>Assumptions!$B$9</f>
@@ -4146,22 +4163,22 @@
       </c>
       <c r="J6" s="115" t="inlineStr">
         <is>
-          <t>Paid Tue 27 Oct. Last run of the month - accrue bonus leave (Checklist step 48). No cash effect.</t>
+          <t>Paid Tue 20 Oct. Last run of the month - accrue bonus leave (Checklist step 48). No cash effect.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>Run 3 - Sat 24 Oct to Fri 6 Nov</t>
+          <t>Run 3 - Sat 17 Oct to Fri 30 Oct</t>
         </is>
       </c>
       <c r="B7" s="128" t="n">
-        <v>46332</v>
+        <v>46325</v>
       </c>
       <c r="C7" s="135">
         <f>Assumptions!$B$16</f>
-        <v>46336</v>
+        <v>46329</v>
       </c>
       <c r="D7" s="136">
         <f>Assumptions!$B$9</f>
@@ -4189,7 +4206,7 @@
       </c>
       <c r="J7" s="115" t="inlineStr">
         <is>
-          <t>Paid Tue 10 Nov - after this forecast, so nothing from it hits the numbers.</t>
+          <t>Paid Tue 3 Nov - lands in week 5.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cash flow: October actuals for weeks 2 to 4 (8 to 28 Oct) from Xero cash P&L and bank
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141HuBtr9dZXPeYR1jN9h28
</commit_message>
<xml_diff>
--- a/cashflow/CTS Cash Flow Forecast - 12102026.xlsx
+++ b/cashflow/CTS Cash Flow Forecast - 12102026.xlsx
@@ -1114,15 +1114,15 @@
       </c>
       <c r="D8" s="10" t="n"/>
       <c r="E8" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="10" t="n"/>
       <c r="G8" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" s="10" t="n"/>
       <c r="I8" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" s="10" t="n"/>
       <c r="K8" s="11" t="n">
@@ -1133,7 +1133,7 @@
       <c r="N8" s="12" t="n"/>
       <c r="O8" s="76" t="inlineStr">
         <is>
-          <t>Week 1 is done and reconciles to Xero (flag 1). Week 2 actuals are in to Mon 12 Oct only - flag stays 0 until the week closes Wed 14 Oct and the bank balance is keyed.</t>
+          <t>Weeks 1 to 4 are done (flag 1). Weeks 2 to 4 are built off the Xero cash P&amp;L, grossed up for GST, with the bank balance worked back from Xero total cash. Week 5 runs to 4 Nov and is in the 29 Oct forecast file.</t>
         </is>
       </c>
     </row>
@@ -1161,27 +1161,27 @@
       </c>
       <c r="F10" s="119">
         <f>IF(E$8=1,E59,D58)</f>
-        <v>263901.67999999993</v>
+        <v>579568.07</v>
       </c>
       <c r="G10" s="119">
         <f>F10</f>
-        <v>263901.67999999993</v>
+        <v>579568.07</v>
       </c>
       <c r="H10" s="119">
         <f>IF(G$8=1,G59,F58)</f>
-        <v>498505.9666666666</v>
+        <v>455481.91000000003</v>
       </c>
       <c r="I10" s="119">
         <f>H10</f>
-        <v>498505.9666666666</v>
+        <v>455481.91000000003</v>
       </c>
       <c r="J10" s="119">
         <f>IF(I$8=1,I59,H58)</f>
-        <v>362388.61933333334</v>
+        <v>439930.67999999993</v>
       </c>
       <c r="K10" s="119">
         <f>J10</f>
-        <v>362388.61933333334</v>
+        <v>439930.67999999993</v>
       </c>
       <c r="L10" s="119">
         <f>B10</f>
@@ -1234,19 +1234,25 @@
         <v>142696.27</v>
       </c>
       <c r="E13" s="121">
-        <f>112683.22+18891.66+9086.39+1661+506+374</f>
-        <v>143202.27000000002</v>
+        <f>ROUND(369617.53*1.1,2)</f>
+        <v>406579.28</v>
       </c>
       <c r="F13" s="120">
         <f>SUMIFS(Receivables!$F$5:$F$65,Receivables!$H$5:$H$65,"&gt;="&amp;Assumptions!$B$46,Receivables!$H$5:$H$65,"&lt;="&amp;Assumptions!$C$46)+Assumptions!$B$39/3</f>
         <v>234604.28666666668</v>
       </c>
-      <c r="G13" s="121" t="n"/>
+      <c r="G13" s="121">
+        <f>ROUND(103182.08*1.1,2)</f>
+        <v>113500.29</v>
+      </c>
       <c r="H13" s="120">
         <f>SUMIFS(Receivables!$F$5:$F$65,Receivables!$H$5:$H$65,"&gt;="&amp;Assumptions!$B$47,Receivables!$H$5:$H$65,"&lt;="&amp;Assumptions!$C$47)+Assumptions!$B$39/3</f>
         <v>12626.466666666667</v>
       </c>
-      <c r="I13" s="121" t="n"/>
+      <c r="I13" s="121">
+        <f>ROUND(17509*1.1,2)</f>
+        <v>19259.9</v>
+      </c>
       <c r="J13" s="120">
         <f>SUMIFS(Receivables!$F$5:$F$65,Receivables!$H$5:$H$65,"&gt;="&amp;Assumptions!$B$48,Receivables!$H$5:$H$65,"&lt;="&amp;Assumptions!$C$48)+Assumptions!$B$39/3</f>
         <v>91870.13666666666</v>
@@ -1258,15 +1264,15 @@
       </c>
       <c r="M13" s="120">
         <f>SUM(C13,E13,G13,I13,K13)</f>
-        <v>301061.4</v>
+        <v>697198.6000000001</v>
       </c>
       <c r="N13" s="120">
         <f>(C13-B13)*C$8+(E13-D13)*E$8+(G13-F13)*G$8+(I13-H13)*I$8+(K13-J13)*K$8</f>
-        <v>23268.21000000002</v>
+        <v>172680.65666666668</v>
       </c>
       <c r="O13" s="108" t="inlineStr">
         <is>
-          <t>Week 1 now includes 6-7 Oct: PwC $9,350, CBA Melb $93.50, APA $627, CBA Bris $8,043.20. Week 2 to 12 Oct: Deloitte $112,683.22 and $18,891.66, CEO Institute $9,086.39, ASX $1,661, Dimensional $506, Ricoh $374. Nothing from Aware yet.</t>
+          <t>Week 2: Aware $225,887 landed Tue 13 Oct, plus Deloitte, CEO Institute, ASX. Week 3: CBA Sep contract invoices (15 Oct), Aware Appspace $23,317, ICC, Bankwest. Week 4: Aware maintenance $12,100 and the Perth USB-C job (27 Oct), RSNSW. All from Xero cash P&amp;L x 1.1.</t>
         </is>
       </c>
     </row>
@@ -1294,12 +1300,16 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="G14" s="121" t="n"/>
+      <c r="G14" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="H14" s="120">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="I14" s="121" t="n"/>
+      <c r="I14" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J14" s="120">
         <f>Assumptions!$B$40</f>
         <v>600</v>
@@ -1343,7 +1353,7 @@
       </c>
       <c r="E15" s="122">
         <f>E13+E14</f>
-        <v>143202.27000000002</v>
+        <v>406579.28</v>
       </c>
       <c r="F15" s="122">
         <f>F13+F14</f>
@@ -1351,7 +1361,7 @@
       </c>
       <c r="G15" s="122">
         <f>G13+G14</f>
-        <v>0</v>
+        <v>113500.29</v>
       </c>
       <c r="H15" s="122">
         <f>H13+H14</f>
@@ -1359,7 +1369,7 @@
       </c>
       <c r="I15" s="122">
         <f>I13+I14</f>
-        <v>0</v>
+        <v>19259.9</v>
       </c>
       <c r="J15" s="122">
         <f>J13+J14</f>
@@ -1375,11 +1385,11 @@
       </c>
       <c r="M15" s="122">
         <f>M13+M14</f>
-        <v>301491.57</v>
+        <v>697628.7700000001</v>
       </c>
       <c r="N15" s="122">
         <f>N13+N14</f>
-        <v>23698.38000000002</v>
+        <v>173110.8266666667</v>
       </c>
       <c r="O15" s="16" t="n"/>
     </row>
@@ -1436,12 +1446,17 @@
         <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$46,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$46)</f>
         <v>85248</v>
       </c>
-      <c r="G19" s="121" t="n"/>
+      <c r="G19" s="121">
+        <f>ROUND(111704.13*Assumptions!$B$10,2)</f>
+        <v>85788.77</v>
+      </c>
       <c r="H19" s="120">
         <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$47,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$47)</f>
         <v>0</v>
       </c>
-      <c r="I19" s="121" t="n"/>
+      <c r="I19" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J19" s="120">
         <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$48,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$48)</f>
         <v>85248</v>
@@ -1453,15 +1468,15 @@
       </c>
       <c r="M19" s="120">
         <f>SUM(C19,E19,G19,I19,K19)</f>
-        <v>79736.05</v>
+        <v>165524.82</v>
       </c>
       <c r="N19" s="120">
         <f>(C19-B19)*C$8+(E19-D19)*E$8+(G19-F19)*G$8+(I19-H19)*I$8+(K19-J19)*K$8</f>
-        <v>-5511.949999999997</v>
+        <v>-4971.179999999993</v>
       </c>
       <c r="O19" s="108" t="inlineStr">
         <is>
-          <t>Payroll tab - gross x net %. Fortnight is Sat to Fri and the money goes out the Tuesday after: Tue 6 Oct (week 1), Tue 20 Oct (week 3) and Tue 3 Nov (week 5). 6 Oct actual is from the Xero bank movement - swap in the ABA figure.</t>
+          <t>Payroll tab - gross x net %. Pay runs Tue 6 Oct (week 1, $79.7k from the bank) and Tue 20 Oct (week 3, $111,704 gross per Xero, net at 78.8% - swap in the ABA figure). Next one Tue 3 Nov is in the new file.</t>
         </is>
       </c>
     </row>
@@ -1489,12 +1504,16 @@
         <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$46,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$46)</f>
         <v>13320</v>
       </c>
-      <c r="G20" s="121" t="n"/>
+      <c r="G20" s="121" t="n">
+        <v>14214.47</v>
+      </c>
       <c r="H20" s="120">
         <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$47,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$47)</f>
         <v>0</v>
       </c>
-      <c r="I20" s="121" t="n"/>
+      <c r="I20" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J20" s="120">
         <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$48,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$48)</f>
         <v>13320</v>
@@ -1506,15 +1525,15 @@
       </c>
       <c r="M20" s="120">
         <f>SUM(C20,E20,G20,I20,K20)</f>
-        <v>13083.54</v>
+        <v>27298.010000000002</v>
       </c>
       <c r="N20" s="120">
         <f>(C20-B20)*C$8+(E20-D20)*E$8+(G20-F20)*G$8+(I20-H20)*I$8+(K20-J20)*K$8</f>
-        <v>-236.45999999999913</v>
+        <v>658.0100000000002</v>
       </c>
       <c r="O20" s="108" t="inlineStr">
         <is>
-          <t>Gross x 12%. EH direct debits it in the pay run week.</t>
+          <t>Gross x 12%. Actuals are the super in the Xero pay run journals ($13,084 on 7 Oct, $14,214 on 21 Oct).</t>
         </is>
       </c>
     </row>
@@ -1540,12 +1559,16 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="G21" s="121" t="n"/>
+      <c r="G21" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="H21" s="120">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="I21" s="121" t="n"/>
+      <c r="I21" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J21" s="120">
         <f>0</f>
         <v>0</v>
@@ -1593,12 +1616,16 @@
         <f>IF(AND(Assumptions!$B$19&gt;=Assumptions!$B$46,Assumptions!$B$19&lt;=Assumptions!$C$46),Assumptions!$B$17+Assumptions!$B$18,0)</f>
         <v>0</v>
       </c>
-      <c r="G22" s="121" t="n"/>
+      <c r="G22" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="H22" s="120">
         <f>IF(AND(Assumptions!$B$19&gt;=Assumptions!$B$47,Assumptions!$B$19&lt;=Assumptions!$C$47),Assumptions!$B$17+Assumptions!$B$18,0)</f>
         <v>0</v>
       </c>
-      <c r="I22" s="121" t="n"/>
+      <c r="I22" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J22" s="120">
         <f>IF(AND(Assumptions!$B$19&gt;=Assumptions!$B$48,Assumptions!$B$19&lt;=Assumptions!$C$48),Assumptions!$B$17+Assumptions!$B$18,0)</f>
         <v>0</v>
@@ -1644,12 +1671,16 @@
         <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$46,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$46)</f>
         <v>1000</v>
       </c>
-      <c r="G23" s="121" t="n"/>
+      <c r="G23" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="H23" s="120">
         <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$47,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$47)</f>
         <v>0</v>
       </c>
-      <c r="I23" s="121" t="n"/>
+      <c r="I23" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J23" s="120">
         <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$48,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$48)</f>
         <v>1000</v>
@@ -1665,7 +1696,7 @@
       </c>
       <c r="N23" s="120">
         <f>(C23-B23)*C$8+(E23-D23)*E$8+(G23-F23)*G$8+(I23-H23)*I$8+(K23-J23)*K$8</f>
-        <v>-1000</v>
+        <v>-2000</v>
       </c>
       <c r="O23" s="108" t="inlineStr">
         <is>
@@ -1701,7 +1732,7 @@
       </c>
       <c r="G24" s="123">
         <f>G19+G20+G21+G22+G23</f>
-        <v>0</v>
+        <v>100003.24</v>
       </c>
       <c r="H24" s="123">
         <f>H19+H20+H21+H22+H23</f>
@@ -1725,11 +1756,11 @@
       </c>
       <c r="M24" s="123">
         <f>M19+M20+M21+M22+M23</f>
-        <v>101422.34</v>
+        <v>201425.58000000002</v>
       </c>
       <c r="N24" s="123">
         <f>N19+N20+N21+N22+N23</f>
-        <v>-7140.659999999996</v>
+        <v>-6705.419999999993</v>
       </c>
       <c r="O24" s="12" t="n"/>
     </row>
@@ -1765,12 +1796,18 @@
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Equipment purchases")+Assumptions!$B$29/5</f>
         <v>4000</v>
       </c>
-      <c r="G27" s="121" t="n"/>
+      <c r="G27" s="121">
+        <f>ROUND(80501.16*1.1,2)</f>
+        <v>88551.28</v>
+      </c>
       <c r="H27" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Equipment purchases")+Assumptions!$B$29/5</f>
         <v>4000</v>
       </c>
-      <c r="I27" s="121" t="n"/>
+      <c r="I27" s="121">
+        <f>ROUND(11382*1.1,2)</f>
+        <v>12520.2</v>
+      </c>
       <c r="J27" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Equipment purchases")+Assumptions!$B$29/5</f>
         <v>4000</v>
@@ -1782,15 +1819,15 @@
       </c>
       <c r="M27" s="120">
         <f>SUM(C27,E27,G27,I27,K27)</f>
-        <v>209729.55</v>
+        <v>310801.02999999997</v>
       </c>
       <c r="N27" s="120">
         <f>(C27-B27)*C$8+(E27-D27)*E$8+(G27-F27)*G$8+(I27-H27)*I$8+(K27-J27)*K$8</f>
-        <v>-28708.199999999983</v>
+        <v>91973.58</v>
       </c>
       <c r="O27" s="108" t="inlineStr">
         <is>
-          <t>139k was paid on the 29/09/2026. Remittance (Complete AV) table  under GC approvals was send on the 29/09. Week 2 to 12 Oct: LiveU SDI/modems $26,004 plus small items ($28,737 ex GST per Xero cash P&amp;L). Complete AV labour and programming $39,033.02 was released and paid 8 Oct - whole bill now paid.</t>
+          <t>139k materials paid 29 Sep, labour $39,033 released and paid 8 Oct. Week 3 actual $88.6k is the equipment purchases in Xero cash P&amp;L 15-21 Oct - a lot bigger than the estimate, worth a look at what it was.</t>
         </is>
       </c>
     </row>
@@ -1817,12 +1854,18 @@
         <f>Assumptions!$B$27/5</f>
         <v>8000</v>
       </c>
-      <c r="G28" s="121" t="n"/>
+      <c r="G28" s="121">
+        <f>ROUND((9090+1628.4)*1.1,2)</f>
+        <v>11790.24</v>
+      </c>
       <c r="H28" s="120">
         <f>Assumptions!$B$27/5</f>
         <v>8000</v>
       </c>
-      <c r="I28" s="121" t="n"/>
+      <c r="I28" s="121">
+        <f>ROUND(3055*1.1,2)</f>
+        <v>3360.5</v>
+      </c>
       <c r="J28" s="120">
         <f>Assumptions!$B$27/5</f>
         <v>8000</v>
@@ -1834,11 +1877,11 @@
       </c>
       <c r="M28" s="120">
         <f>SUM(C28,E28,G28,I28,K28)</f>
-        <v>9510.18</v>
+        <v>24660.92</v>
       </c>
       <c r="N28" s="120">
         <f>(C28-B28)*C$8+(E28-D28)*E$8+(G28-F28)*G$8+(I28-H28)*I$8+(K28-J28)*K$8</f>
-        <v>-8000</v>
+        <v>-7339.08</v>
       </c>
       <c r="O28" s="108" t="inlineStr">
         <is>
@@ -1869,12 +1912,18 @@
         <f>Assumptions!$B$28/5</f>
         <v>6000</v>
       </c>
-      <c r="G29" s="121" t="n"/>
+      <c r="G29" s="121">
+        <f>ROUND((4167.5+42.5+9.73)*1.1,2)</f>
+        <v>4641.7</v>
+      </c>
       <c r="H29" s="120">
         <f>Assumptions!$B$28/5</f>
         <v>6000</v>
       </c>
-      <c r="I29" s="121" t="n"/>
+      <c r="I29" s="121">
+        <f>ROUND((2630+43.75)*1.1,2)</f>
+        <v>2941.13</v>
+      </c>
       <c r="J29" s="120">
         <f>Assumptions!$B$28/5</f>
         <v>6000</v>
@@ -1886,11 +1935,11 @@
       </c>
       <c r="M29" s="120">
         <f>SUM(C29,E29,G29,I29,K29)</f>
-        <v>15724.52</v>
+        <v>23307.350000000002</v>
       </c>
       <c r="N29" s="120">
         <f>(C29-B29)*C$8+(E29-D29)*E$8+(G29-F29)*G$8+(I29-H29)*I$8+(K29-J29)*K$8</f>
-        <v>-6000</v>
+        <v>-692.6499999999996</v>
       </c>
       <c r="O29" s="108" t="inlineStr">
         <is>
@@ -1914,19 +1963,23 @@
         <v>5712.04</v>
       </c>
       <c r="E30" s="121">
-        <f>ROUND(18837.31*1.1,2)</f>
-        <v>20721.04</v>
+        <f>ROUND(19053.3*1.1,2)</f>
+        <v>20958.63</v>
       </c>
       <c r="F30" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Client subscriptions")+Assumptions!$B$31/5</f>
         <v>600</v>
       </c>
-      <c r="G30" s="121" t="n"/>
+      <c r="G30" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="H30" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Client subscriptions")+Assumptions!$B$31/5</f>
         <v>600</v>
       </c>
-      <c r="I30" s="121" t="n"/>
+      <c r="I30" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J30" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Client subscriptions")+Assumptions!$B$31/5</f>
         <v>600</v>
@@ -1938,11 +1991,11 @@
       </c>
       <c r="M30" s="120">
         <f>SUM(C30,E30,G30,I30,K30)</f>
-        <v>20721.04</v>
+        <v>20958.63</v>
       </c>
       <c r="N30" s="120">
         <f>(C30-B30)*C$8+(E30-D30)*E$8+(G30-F30)*G$8+(I30-H30)*I$8+(K30-J30)*K$8</f>
-        <v>-6328.8</v>
+        <v>7717.790000000001</v>
       </c>
       <c r="O30" s="108" t="inlineStr">
         <is>
@@ -1966,19 +2019,25 @@
         <v>1400</v>
       </c>
       <c r="E31" s="121">
-        <f>ROUND((1115.04+46.69)*1.1,2)</f>
-        <v>1277.9</v>
+        <f>ROUND((1115.04+560.9+46.69)*1.1,2)</f>
+        <v>1894.89</v>
       </c>
       <c r="F31" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Direct travel &amp; freight")+Assumptions!$B$30/5</f>
         <v>1400</v>
       </c>
-      <c r="G31" s="121" t="n"/>
+      <c r="G31" s="121">
+        <f>ROUND((2525.5+2214.76+1132+834.55)*1.1,2)</f>
+        <v>7377.49</v>
+      </c>
       <c r="H31" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Direct travel &amp; freight")+Assumptions!$B$30/5</f>
         <v>1400</v>
       </c>
-      <c r="I31" s="121" t="n"/>
+      <c r="I31" s="121">
+        <f>ROUND((658+361.82)*1.1,2)</f>
+        <v>1121.8</v>
+      </c>
       <c r="J31" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Direct travel &amp; freight")+Assumptions!$B$30/5</f>
         <v>1400</v>
@@ -1990,11 +2049,11 @@
       </c>
       <c r="M31" s="120">
         <f>SUM(C31,E31,G31,I31,K31)</f>
-        <v>1277.9</v>
+        <v>10394.179999999998</v>
       </c>
       <c r="N31" s="120">
         <f>(C31-B31)*C$8+(E31-D31)*E$8+(G31-F31)*G$8+(I31-H31)*I$8+(K31-J31)*K$8</f>
-        <v>-1400</v>
+        <v>4794.18</v>
       </c>
       <c r="O31" s="108" t="inlineStr">
         <is>
@@ -2022,7 +2081,7 @@
       </c>
       <c r="E32" s="123">
         <f>E27+E28+E29+E30+E31</f>
-        <v>117876.95999999999</v>
+        <v>118731.54000000001</v>
       </c>
       <c r="F32" s="123">
         <f>F27+F28+F29+F30+F31</f>
@@ -2030,7 +2089,7 @@
       </c>
       <c r="G32" s="123">
         <f>G27+G28+G29+G30+G31</f>
-        <v>0</v>
+        <v>112360.71</v>
       </c>
       <c r="H32" s="123">
         <f>H27+H28+H29+H30+H31</f>
@@ -2038,7 +2097,7 @@
       </c>
       <c r="I32" s="123">
         <f>I27+I28+I29+I30+I31</f>
-        <v>0</v>
+        <v>19943.63</v>
       </c>
       <c r="J32" s="123">
         <f>J27+J28+J29+J30+J31</f>
@@ -2054,11 +2113,11 @@
       </c>
       <c r="M32" s="123">
         <f>M27+M28+M29+M30+M31</f>
-        <v>256963.18999999997</v>
+        <v>390122.1099999999</v>
       </c>
       <c r="N32" s="123">
         <f>N27+N28+N29+N30+N31</f>
-        <v>-50436.999999999985</v>
+        <v>96453.82</v>
       </c>
       <c r="O32" s="12" t="n"/>
     </row>
@@ -2091,12 +2150,16 @@
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Rent")</f>
         <v>0</v>
       </c>
-      <c r="G35" s="121" t="n"/>
+      <c r="G35" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="H35" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Rent")</f>
         <v>0</v>
       </c>
-      <c r="I35" s="121" t="n"/>
+      <c r="I35" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J35" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Rent")</f>
         <v>0</v>
@@ -2142,12 +2205,17 @@
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"IT support")</f>
         <v>0</v>
       </c>
-      <c r="G36" s="121" t="n"/>
+      <c r="G36" s="121">
+        <f>ROUND(9178.55*1.1,2)</f>
+        <v>10096.41</v>
+      </c>
       <c r="H36" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"IT support")</f>
         <v>0</v>
       </c>
-      <c r="I36" s="121" t="n"/>
+      <c r="I36" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J36" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"IT support")</f>
         <v>0</v>
@@ -2159,11 +2227,11 @@
       </c>
       <c r="M36" s="120">
         <f>SUM(C36,E36,G36,I36,K36)</f>
-        <v>0</v>
+        <v>10096.41</v>
       </c>
       <c r="N36" s="120">
         <f>(C36-B36)*C$8+(E36-D36)*E$8+(G36-F36)*G$8+(I36-H36)*I$8+(K36-J36)*K$8</f>
-        <v>0</v>
+        <v>10096.41</v>
       </c>
       <c r="O36" s="108" t="inlineStr">
         <is>
@@ -2193,12 +2261,18 @@
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Advertising")</f>
         <v>0</v>
       </c>
-      <c r="G37" s="121" t="n"/>
+      <c r="G37" s="121">
+        <f>ROUND(4250*1.1,2)</f>
+        <v>4675</v>
+      </c>
       <c r="H37" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Advertising")</f>
         <v>0</v>
       </c>
-      <c r="I37" s="121" t="n"/>
+      <c r="I37" s="121">
+        <f>ROUND(4385*1.1,2)</f>
+        <v>4823.5</v>
+      </c>
       <c r="J37" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Advertising")</f>
         <v>0</v>
@@ -2210,11 +2284,11 @@
       </c>
       <c r="M37" s="120">
         <f>SUM(C37,E37,G37,I37,K37)</f>
-        <v>0</v>
+        <v>9498.5</v>
       </c>
       <c r="N37" s="120">
         <f>(C37-B37)*C$8+(E37-D37)*E$8+(G37-F37)*G$8+(I37-H37)*I$8+(K37-J37)*K$8</f>
-        <v>-6600</v>
+        <v>2898.5</v>
       </c>
       <c r="O37" s="108" t="inlineStr">
         <is>
@@ -2246,12 +2320,16 @@
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Professional fees")+Assumptions!$B$33/5</f>
         <v>4650</v>
       </c>
-      <c r="G38" s="121" t="n"/>
+      <c r="G38" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="H38" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Professional fees")+Assumptions!$B$33/5</f>
         <v>800</v>
       </c>
-      <c r="I38" s="121" t="n"/>
+      <c r="I38" s="121" t="n">
+        <v>342</v>
+      </c>
       <c r="J38" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Professional fees")+Assumptions!$B$33/5</f>
         <v>800</v>
@@ -2263,11 +2341,11 @@
       </c>
       <c r="M38" s="120">
         <f>SUM(C38,E38,G38,I38,K38)</f>
-        <v>880</v>
+        <v>1222</v>
       </c>
       <c r="N38" s="120">
         <f>(C38-B38)*C$8+(E38-D38)*E$8+(G38-F38)*G$8+(I38-H38)*I$8+(K38-J38)*K$8</f>
-        <v>-800</v>
+        <v>-6708</v>
       </c>
       <c r="O38" s="108" t="inlineStr">
         <is>
@@ -2290,19 +2368,25 @@
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Dues &amp; subscriptions")</f>
         <v>0</v>
       </c>
-      <c r="E39" s="121" t="n">
-        <v>0</v>
+      <c r="E39" s="121">
+        <f>ROUND(629.85*1.1,2)</f>
+        <v>692.84</v>
       </c>
       <c r="F39" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Dues &amp; subscriptions")</f>
         <v>2310</v>
       </c>
-      <c r="G39" s="121" t="n"/>
+      <c r="G39" s="121">
+        <f>ROUND(3154.18*1.1,2)</f>
+        <v>3469.6</v>
+      </c>
       <c r="H39" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Dues &amp; subscriptions")</f>
         <v>0</v>
       </c>
-      <c r="I39" s="121" t="n"/>
+      <c r="I39" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J39" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Dues &amp; subscriptions")</f>
         <v>0</v>
@@ -2314,11 +2398,11 @@
       </c>
       <c r="M39" s="120">
         <f>SUM(C39,E39,G39,I39,K39)</f>
-        <v>0</v>
+        <v>4162.44</v>
       </c>
       <c r="N39" s="120">
         <f>(C39-B39)*C$8+(E39-D39)*E$8+(G39-F39)*G$8+(I39-H39)*I$8+(K39-J39)*K$8</f>
-        <v>0</v>
+        <v>1852.44</v>
       </c>
       <c r="O39" s="108" t="inlineStr">
         <is>
@@ -2349,12 +2433,17 @@
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Telephone &amp; internet")</f>
         <v>0</v>
       </c>
-      <c r="G40" s="121" t="n"/>
+      <c r="G40" s="121">
+        <f>ROUND(92*1.1,2)</f>
+        <v>101.2</v>
+      </c>
       <c r="H40" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Telephone &amp; internet")</f>
         <v>0</v>
       </c>
-      <c r="I40" s="121" t="n"/>
+      <c r="I40" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J40" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Telephone &amp; internet")</f>
         <v>0</v>
@@ -2366,11 +2455,11 @@
       </c>
       <c r="M40" s="120">
         <f>SUM(C40,E40,G40,I40,K40)</f>
-        <v>940.11</v>
+        <v>1041.31</v>
       </c>
       <c r="N40" s="120">
         <f>(C40-B40)*C$8+(E40-D40)*E$8+(G40-F40)*G$8+(I40-H40)*I$8+(K40-J40)*K$8</f>
-        <v>0</v>
+        <v>101.2</v>
       </c>
       <c r="O40" s="108" t="inlineStr">
         <is>
@@ -2400,12 +2489,17 @@
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Recruitment")+Assumptions!$B$32/5</f>
         <v>1000</v>
       </c>
-      <c r="G41" s="121" t="n"/>
+      <c r="G41" s="121">
+        <f>ROUND(906*1.1,2)</f>
+        <v>996.6</v>
+      </c>
       <c r="H41" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Recruitment")+Assumptions!$B$32/5</f>
         <v>1000</v>
       </c>
-      <c r="I41" s="121" t="n"/>
+      <c r="I41" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J41" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Recruitment")+Assumptions!$B$32/5</f>
         <v>1000</v>
@@ -2417,11 +2511,11 @@
       </c>
       <c r="M41" s="120">
         <f>SUM(C41,E41,G41,I41,K41)</f>
-        <v>0</v>
+        <v>996.6</v>
       </c>
       <c r="N41" s="120">
         <f>(C41-B41)*C$8+(E41-D41)*E$8+(G41-F41)*G$8+(I41-H41)*I$8+(K41-J41)*K$8</f>
-        <v>-1000</v>
+        <v>-3003.4</v>
       </c>
       <c r="O41" s="108" t="inlineStr">
         <is>
@@ -2451,12 +2545,16 @@
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Insurance")+Assumptions!$B$34/5</f>
         <v>0</v>
       </c>
-      <c r="G42" s="121" t="n"/>
+      <c r="G42" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="H42" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Insurance")+Assumptions!$B$34/5</f>
         <v>0</v>
       </c>
-      <c r="I42" s="121" t="n"/>
+      <c r="I42" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J42" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Insurance")+Assumptions!$B$34/5</f>
         <v>0</v>
@@ -2476,7 +2574,7 @@
       </c>
       <c r="O42" s="108" t="inlineStr">
         <is>
-          <t>Brookvale annual renewals $66,239 due Wed 14 Oct (six bills, GC approved) - Payables tab. Was a $3k a month estimate, now nil on top.</t>
+          <t>Brookvale $66,239 was in the week 2 forecast but has not been paid - still open in Xero at 29 Oct, due 30 Oct. It is in the 2 Nov creditors run in the new file.</t>
         </is>
       </c>
     </row>
@@ -2504,12 +2602,17 @@
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Office")+Assumptions!$B$35/5</f>
         <v>400</v>
       </c>
-      <c r="G43" s="121" t="n"/>
+      <c r="G43" s="121">
+        <f>ROUND((44.04+31.82+27.93+12.95+6.1)*1.1,2)</f>
+        <v>135.12</v>
+      </c>
       <c r="H43" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Office")+Assumptions!$B$35/5</f>
         <v>400</v>
       </c>
-      <c r="I43" s="121" t="n"/>
+      <c r="I43" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J43" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Office")+Assumptions!$B$35/5</f>
         <v>400</v>
@@ -2521,11 +2624,11 @@
       </c>
       <c r="M43" s="120">
         <f>SUM(C43,E43,G43,I43,K43)</f>
-        <v>480.6</v>
+        <v>615.72</v>
       </c>
       <c r="N43" s="120">
         <f>(C43-B43)*C$8+(E43-D43)*E$8+(G43-F43)*G$8+(I43-H43)*I$8+(K43-J43)*K$8</f>
-        <v>-400</v>
+        <v>-1464.88</v>
       </c>
       <c r="O43" s="108" t="inlineStr">
         <is>
@@ -2555,12 +2658,16 @@
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Electricity")</f>
         <v>0</v>
       </c>
-      <c r="G44" s="121" t="n"/>
+      <c r="G44" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="H44" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Electricity")</f>
         <v>0</v>
       </c>
-      <c r="I44" s="121" t="n"/>
+      <c r="I44" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J44" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Electricity")</f>
         <v>0</v>
@@ -2608,12 +2715,17 @@
         <f>Assumptions!$B$36/5</f>
         <v>200</v>
       </c>
-      <c r="G45" s="121" t="n"/>
+      <c r="G45" s="121">
+        <f>ROUND(139.89*1.1,2)+36.86</f>
+        <v>190.74</v>
+      </c>
       <c r="H45" s="120">
         <f>Assumptions!$B$36/5</f>
         <v>200</v>
       </c>
-      <c r="I45" s="121" t="n"/>
+      <c r="I45" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J45" s="120">
         <f>Assumptions!$B$36/5</f>
         <v>200</v>
@@ -2625,11 +2737,11 @@
       </c>
       <c r="M45" s="120">
         <f>SUM(C45,E45,G45,I45,K45)</f>
-        <v>10</v>
+        <v>200.74</v>
       </c>
       <c r="N45" s="120">
         <f>(C45-B45)*C$8+(E45-D45)*E$8+(G45-F45)*G$8+(I45-H45)*I$8+(K45-J45)*K$8</f>
-        <v>-190</v>
+        <v>-599.26</v>
       </c>
       <c r="O45" s="108" t="inlineStr">
         <is>
@@ -2661,12 +2773,16 @@
         <f>Assumptions!$B$37/5</f>
         <v>5000</v>
       </c>
-      <c r="G46" s="121" t="n"/>
+      <c r="G46" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="H46" s="120">
         <f>Assumptions!$B$37/5</f>
         <v>5000</v>
       </c>
-      <c r="I46" s="121" t="n"/>
+      <c r="I46" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J46" s="120">
         <f>Assumptions!$B$37/5</f>
         <v>5000</v>
@@ -2682,11 +2798,11 @@
       </c>
       <c r="N46" s="120">
         <f>(C46-B46)*C$8+(E46-D46)*E$8+(G46-F46)*G$8+(I46-H46)*I$8+(K46-J46)*K$8</f>
-        <v>5000</v>
+        <v>-10000</v>
       </c>
       <c r="O46" s="108" t="inlineStr">
         <is>
-          <t>~$25k a month transferred to the PL and DL cards. Covers every Card row on the Payables tab (subscriptions, travel, electricity, Seek, Goget, EH). Week 1 actual: $10,000 moved to the PL card 7 Oct.</t>
+          <t>~$25k a month to the PL and DL cards. Weeks 2 to 4 actuals are nil here because the card spend is already inside the category lines (Xero cash P&amp;L includes what the cards paid). Only the $10k transfer on 7 Oct is shown, in week 1.</t>
         </is>
       </c>
     </row>
@@ -2712,12 +2828,17 @@
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Other")</f>
         <v>0</v>
       </c>
-      <c r="G47" s="121" t="n"/>
+      <c r="G47" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="H47" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Other")</f>
         <v>0</v>
       </c>
-      <c r="I47" s="121" t="n"/>
+      <c r="I47" s="121">
+        <f>ROUND(360*1.1,2)</f>
+        <v>396</v>
+      </c>
       <c r="J47" s="120">
         <f>SUMIFS(Payables!$D$19:$D$75,Payables!$K$19:$K$75,"Yes",Payables!$G$19:$G$75,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$75,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$75,"&lt;&gt;Card",Payables!$F$19:$F$75,"Other")</f>
         <v>0</v>
@@ -2729,11 +2850,11 @@
       </c>
       <c r="M47" s="120">
         <f>SUM(C47,E47,G47,I47,K47)</f>
-        <v>0</v>
+        <v>396</v>
       </c>
       <c r="N47" s="120">
         <f>(C47-B47)*C$8+(E47-D47)*E$8+(G47-F47)*G$8+(I47-H47)*I$8+(K47-J47)*K$8</f>
-        <v>0</v>
+        <v>396</v>
       </c>
       <c r="O47" s="108" t="inlineStr">
         <is>
@@ -2758,17 +2879,23 @@
         <f>IF('Creditors Run'!$B$5=1,SUMPRODUCT(('Creditors Run'!$A$11:$A$510&lt;&gt;"")*ISNUMBER('Creditors Run'!$I$11:$I$510)*('Creditors Run'!$M$11:$M$510="")*('Creditors Run'!$N$11:$N$510&gt;=Assumptions!$B$45)*('Creditors Run'!$N$11:$N$510&lt;=Assumptions!$C$45),'Creditors Run'!$I$11:$I$510),0)</f>
         <v>67811.82</v>
       </c>
-      <c r="E48" s="121" t="n"/>
+      <c r="E48" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="F48" s="120">
         <f>IF('Creditors Run'!$B$5=1,SUMPRODUCT(('Creditors Run'!$A$11:$A$510&lt;&gt;"")*ISNUMBER('Creditors Run'!$I$11:$I$510)*('Creditors Run'!$M$11:$M$510="")*('Creditors Run'!$N$11:$N$510&gt;=Assumptions!$B$46)*('Creditors Run'!$N$11:$N$510&lt;=Assumptions!$C$46),'Creditors Run'!$I$11:$I$510),0)</f>
         <v>26442.059999999998</v>
       </c>
-      <c r="G48" s="121" t="n"/>
+      <c r="G48" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="H48" s="120">
         <f>IF('Creditors Run'!$B$5=1,SUMPRODUCT(('Creditors Run'!$A$11:$A$510&lt;&gt;"")*ISNUMBER('Creditors Run'!$I$11:$I$510)*('Creditors Run'!$M$11:$M$510="")*('Creditors Run'!$N$11:$N$510&gt;=Assumptions!$B$47)*('Creditors Run'!$N$11:$N$510&lt;=Assumptions!$C$47),'Creditors Run'!$I$11:$I$510),0)</f>
         <v>20985.43</v>
       </c>
-      <c r="I48" s="121" t="n"/>
+      <c r="I48" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J48" s="120">
         <f>IF('Creditors Run'!$B$5=1,SUMPRODUCT(('Creditors Run'!$A$11:$A$510&lt;&gt;"")*ISNUMBER('Creditors Run'!$I$11:$I$510)*('Creditors Run'!$M$11:$M$510="")*('Creditors Run'!$N$11:$N$510&gt;=Assumptions!$B$48)*('Creditors Run'!$N$11:$N$510&lt;=Assumptions!$C$48),'Creditors Run'!$I$11:$I$510),0)</f>
         <v>25592.92</v>
@@ -2784,11 +2911,11 @@
       </c>
       <c r="N48" s="120">
         <f>(C48-B48)*C$8+(E48-D48)*E$8+(G48-F48)*G$8+(I48-H48)*I$8+(K48-J48)*K$8</f>
-        <v>77302.54</v>
+        <v>-37936.77000000001</v>
       </c>
       <c r="O48" s="108" t="inlineStr">
         <is>
-          <t>Creditors Run tab - paste the Xero aged payables detail in each month and it lands here on the run date (or the date in column L). Week 1 actual is the 1 Oct run. The Payables tab's Xero bill rows drop out of the lines above while this is switched on, so nothing is double counted.</t>
+          <t>Creditors Run tab. Week 1 actual is the 1 Oct run ($77,303). No run in weeks 2 to 4 - bills were paid one by one and sit in their category lines.</t>
         </is>
       </c>
     </row>
@@ -2812,7 +2939,7 @@
       </c>
       <c r="E49" s="123">
         <f>E35+E36+E37+E38+E39+E40+E41+E42+E43+E44+E45+E46+E47+E48</f>
-        <v>1185.1100000000001</v>
+        <v>1877.95</v>
       </c>
       <c r="F49" s="123">
         <f>F35+F36+F37+F38+F39+F40+F41+F42+F43+F44+F45+F46+F47+F48</f>
@@ -2820,7 +2947,7 @@
       </c>
       <c r="G49" s="123">
         <f>G35+G36+G37+G38+G39+G40+G41+G42+G43+G44+G45+G46+G47+G48</f>
-        <v>0</v>
+        <v>19664.67</v>
       </c>
       <c r="H49" s="123">
         <f>H35+H36+H37+H38+H39+H40+H41+H42+H43+H44+H45+H46+H47+H48</f>
@@ -2828,7 +2955,7 @@
       </c>
       <c r="I49" s="123">
         <f>I35+I36+I37+I38+I39+I40+I41+I42+I43+I44+I45+I46+I47+I48</f>
-        <v>0</v>
+        <v>5561.5</v>
       </c>
       <c r="J49" s="123">
         <f>J35+J36+J37+J38+J39+J40+J41+J42+J43+J44+J45+J46+J47+J48</f>
@@ -2844,11 +2971,11 @@
       </c>
       <c r="M49" s="123">
         <f>M35+M36+M37+M38+M39+M40+M41+M42+M43+M44+M45+M46+M47+M48</f>
-        <v>89613.25</v>
+        <v>115532.26</v>
       </c>
       <c r="N49" s="123">
         <f>N35+N36+N37+N38+N39+N40+N41+N42+N43+N44+N45+N46+N47+N48</f>
-        <v>73312.54</v>
+        <v>-44367.76000000001</v>
       </c>
       <c r="O49" s="12" t="n"/>
     </row>
@@ -2881,12 +3008,16 @@
         <f>IF(AND(Assumptions!$B$25&gt;=Assumptions!$B$46,Assumptions!$B$25&lt;=Assumptions!$C$46),Assumptions!$B$21*(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24),0)</f>
         <v>0</v>
       </c>
-      <c r="G52" s="121" t="n"/>
+      <c r="G52" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="H52" s="120">
         <f>IF(AND(Assumptions!$B$25&gt;=Assumptions!$B$47,Assumptions!$B$25&lt;=Assumptions!$C$47),Assumptions!$B$21*(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24),0)</f>
         <v>100358.38399999999</v>
       </c>
-      <c r="I52" s="121" t="n"/>
+      <c r="I52" s="121" t="n">
+        <v>0</v>
+      </c>
       <c r="J52" s="120">
         <f>IF(AND(Assumptions!$B$25&gt;=Assumptions!$B$48,Assumptions!$B$25&lt;=Assumptions!$C$48),Assumptions!$B$21*(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24),0)</f>
         <v>0</v>
@@ -2902,11 +3033,11 @@
       </c>
       <c r="N52" s="120">
         <f>(C52-B52)*C$8+(E52-D52)*E$8+(G52-F52)*G$8+(I52-H52)*I$8+(K52-J52)*K$8</f>
-        <v>0</v>
+        <v>-100358.38399999999</v>
       </c>
       <c r="O52" s="108" t="str">
-        <f>"Q1 BAS est. "&amp;TEXT(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24,"$#,##0")&amp;" (Sep PAYG "&amp;TEXT(Assumptions!$B$22,"$#,##0")&amp;" + GST est "&amp;TEXT(Assumptions!$B$23,"$#,##0")&amp;" + instalment "&amp;TEXT(Assumptions!$B$24,"$#,##0")&amp;"), due "&amp;TEXT(Assumptions!$B$25,"d mmm")&amp;". Toggle on Assumptions = "&amp;Assumptions!$B$21&amp;" (1 = in the forecast)."</f>
-        <v>Q1 BAS est. $100,358 (Sep PAYG $50,358 + GST est $50,000 + instalment $0,), due 28 Oct. Toggle on Assumptions = 1 (1 = in the forecast).</v>
+        <f>"Q1 BAS est. "&amp;TEXT(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24,"$#,##0")&amp;" was in week 4 (28 Oct) but did not go out - Xero bank is flat 28 to 29 Oct. Carried into the 29 Oct forecast as 25 Nov through the agent."</f>
+        <v>Q1 BAS est. $100,358 was in week 4 (28 Oct) but did not go out - Xero bank is flat 28 to 29 Oct. Carried into the 29 Oct forecast as 25 Nov through the agent.</v>
       </c>
     </row>
     <row r="53">
@@ -2965,7 +3096,7 @@
       </c>
       <c r="N53" s="123">
         <f>N52</f>
-        <v>0</v>
+        <v>-100358.38399999999</v>
       </c>
       <c r="O53" s="12" t="n"/>
     </row>
@@ -2989,7 +3120,7 @@
       </c>
       <c r="E55" s="122">
         <f>E24+E32+E49+E53</f>
-        <v>119062.06999999999</v>
+        <v>120609.49</v>
       </c>
       <c r="F55" s="122">
         <f>F24+F32+F49+F66</f>
@@ -2997,7 +3128,7 @@
       </c>
       <c r="G55" s="122">
         <f>G24+G32+G49+G53</f>
-        <v>0</v>
+        <v>232028.62</v>
       </c>
       <c r="H55" s="122">
         <f>H24+H32+H49+H53</f>
@@ -3005,7 +3136,7 @@
       </c>
       <c r="I55" s="122">
         <f>I24+I32+I49+I53</f>
-        <v>0</v>
+        <v>25505.13</v>
       </c>
       <c r="J55" s="122">
         <f>J24+J32+J49+J53</f>
@@ -3021,11 +3152,11 @@
       </c>
       <c r="M55" s="122">
         <f>M24+M32+M49+M53</f>
-        <v>447998.77999999997</v>
+        <v>707079.95</v>
       </c>
       <c r="N55" s="122">
         <f>N24+N32+N49+N53</f>
-        <v>15734.880000000012</v>
+        <v>-54977.74399999999</v>
       </c>
       <c r="O55" s="16" t="n"/>
     </row>
@@ -3049,7 +3180,7 @@
       </c>
       <c r="E57" s="122">
         <f>E15-E55</f>
-        <v>24140.200000000026</v>
+        <v>285969.79000000004</v>
       </c>
       <c r="F57" s="122">
         <f>F15-F68</f>
@@ -3057,7 +3188,7 @@
       </c>
       <c r="G57" s="122">
         <f>G15-G55</f>
-        <v>0</v>
+        <v>-118528.33</v>
       </c>
       <c r="H57" s="122">
         <f>H15-H55</f>
@@ -3065,7 +3196,7 @@
       </c>
       <c r="I57" s="122">
         <f>I15-I55</f>
-        <v>0</v>
+        <v>-6245.23</v>
       </c>
       <c r="J57" s="122">
         <f>J15-J55</f>
@@ -3081,11 +3212,11 @@
       </c>
       <c r="M57" s="122">
         <f>M15-M55</f>
-        <v>-146507.20999999996</v>
+        <v>-9451.179999999818</v>
       </c>
       <c r="N57" s="122">
         <f>N15-N55</f>
-        <v>7963.500000000007</v>
+        <v>228088.57066666667</v>
       </c>
       <c r="O57" s="16" t="n"/>
     </row>
@@ -3107,29 +3238,29 @@
         <f>D10+D57</f>
         <v>263901.67999999993</v>
       </c>
-      <c r="E58" s="125" t="str">
+      <c r="E58" s="125">
         <f>IF(E$8=1,E10+E57,"")</f>
-        <v/>
+        <v>547717.19</v>
       </c>
       <c r="F58" s="125">
         <f>F10+F57</f>
-        <v>498505.9666666666</v>
-      </c>
-      <c r="G58" s="125" t="str">
+        <v>814172.3566666667</v>
+      </c>
+      <c r="G58" s="125">
         <f>IF(G$8=1,G10+G57,"")</f>
-        <v/>
+        <v>461039.73999999993</v>
       </c>
       <c r="H58" s="125">
         <f>H10+H57</f>
-        <v>362388.61933333334</v>
-      </c>
-      <c r="I58" s="125" t="str">
+        <v>319364.5626666667</v>
+      </c>
+      <c r="I58" s="125">
         <f>IF(I$8=1,I10+I57,"")</f>
-        <v/>
+        <v>449236.68000000005</v>
       </c>
       <c r="J58" s="125">
         <f>J10+J57</f>
-        <v>302297.836</v>
+        <v>379839.8966666666</v>
       </c>
       <c r="K58" s="125" t="str">
         <f>IF(K$8=1,K10+K57,"")</f>
@@ -3137,11 +3268,11 @@
       </c>
       <c r="L58" s="125">
         <f>J58</f>
-        <v>302297.836</v>
+        <v>379839.8966666666</v>
       </c>
       <c r="M58" s="125">
         <f>IF(K$8=1,K58,IF(I$8=1,I58,IF(G$8=1,G58,IF(E$8=1,E58,IF(C$8=1,C58,"")))))</f>
-        <v>264507.58999999997</v>
+        <v>449236.68000000005</v>
       </c>
       <c r="N58" s="26" t="n"/>
       <c r="O58" s="78" t="inlineStr">
@@ -3162,11 +3293,20 @@
         <v>261747.39999999997</v>
       </c>
       <c r="D59" s="10" t="n"/>
-      <c r="E59" s="121" t="n"/>
+      <c r="E59" s="121">
+        <f>1036314.34-456746.27</f>
+        <v>579568.07</v>
+      </c>
       <c r="F59" s="10" t="n"/>
-      <c r="G59" s="121" t="n"/>
+      <c r="G59" s="121">
+        <f>912228.18-456746.27</f>
+        <v>455481.91000000003</v>
+      </c>
       <c r="H59" s="10" t="n"/>
-      <c r="I59" s="121" t="n"/>
+      <c r="I59" s="121">
+        <f>896676.95-456746.27</f>
+        <v>439930.67999999993</v>
+      </c>
       <c r="J59" s="10" t="n"/>
       <c r="K59" s="121" t="n"/>
       <c r="L59" s="12" t="n"/>
@@ -3174,7 +3314,7 @@
       <c r="N59" s="12" t="n"/>
       <c r="O59" s="79" t="inlineStr">
         <is>
-          <t>Type the real closing balance (cheque + savings) in at the end of each week. Week 1 is worked back from Xero: $358,696.23 at Mon 5 Oct, less the $86,948.83 Xero cash drop over 6-7 Oct and the $10k card transfer - replace with the CommBiz 7 Oct figure. Week 2 - key it Wed 14 Oct, then set the flag to 1.</t>
+          <t>Weeks 2 to 4 are worked back from Xero total cash less the other accounts ($456,746, the gap on 5 Oct). Replace each with the CommBiz cheque + savings figure at 14, 21 and 28 Oct. Week 1 is the same method off 7 Oct.</t>
         </is>
       </c>
     </row>
@@ -3190,19 +3330,19 @@
         <v>2760.1900000000023</v>
       </c>
       <c r="D60" s="10" t="n"/>
-      <c r="E60" s="126" t="str">
+      <c r="E60" s="126">
         <f>IF(E$8=1,E58-E59,"")</f>
-        <v/>
+        <v>-31850.880000000005</v>
       </c>
       <c r="F60" s="10" t="n"/>
-      <c r="G60" s="126" t="str">
+      <c r="G60" s="126">
         <f>IF(G$8=1,G58-G59,"")</f>
-        <v/>
+        <v>5557.8299999999</v>
       </c>
       <c r="H60" s="10" t="n"/>
-      <c r="I60" s="126" t="str">
+      <c r="I60" s="126">
         <f>IF(I$8=1,I58-I59,"")</f>
-        <v/>
+        <v>9306.000000000116</v>
       </c>
       <c r="J60" s="10" t="n"/>
       <c r="K60" s="126" t="str">
@@ -3214,7 +3354,7 @@
       <c r="N60" s="12" t="n"/>
       <c r="O60" s="76" t="inlineStr">
         <is>
-          <t>Should be nil once everything's in. Week 1 is about $2.8k unexplained - small card / bank items on 6-7 Oct that aren't on a bill. Clears when the real 7 Oct balance goes in.</t>
+          <t>Should be nil once everything's in. Weeks 2 to 4 show the gap between the Xero P&amp;L method and the bank - card spend, transfers and anything not on a bill. The CommBiz balances will tighten it.</t>
         </is>
       </c>
     </row>
@@ -3283,15 +3423,15 @@
       </c>
       <c r="F64" s="127">
         <f>IF(Payroll!$I$5=0,0,F58/(Payroll!$I$5/2))</f>
-        <v>10.013377122502543</v>
+        <v>16.354096831646046</v>
       </c>
       <c r="H64" s="127">
         <f>IF(Payroll!$I$5=0,0,H58/(Payroll!$I$5/2))</f>
-        <v>7.279218611066474</v>
+        <v>6.415004070919707</v>
       </c>
       <c r="J64" s="127">
         <f>IF(Payroll!$I$5=0,0,J58/(Payroll!$I$5/2))</f>
-        <v>6.072188574642456</v>
+        <v>7.629758490010176</v>
       </c>
       <c r="O64" s="108" t="n"/>
     </row>
@@ -3351,7 +3491,7 @@
     <row r="69" ht="15.75" customHeight="1" s="109">
       <c r="A69" s="110" t="inlineStr">
         <is>
-          <t>1. Aware Super $225,887 (INV-10596) is the big one - still not paid at 12 Oct and now expected 9 Nov, after this forecast. The whole Complete AV bill ($178,119) is now paid ahead of it (materials 29 Sep, labour 8 Oct), so we watch the cheque account until Aware pay. Build-up on the Complete AV tab.</t>
+          <t>1. Aware Super paid the $225,887 on 13 Oct and everything else by 27 Oct - risk cleared. The whole Complete AV bill ($178,119) went out ahead of it. Build-up on the Complete AV tab.</t>
         </is>
       </c>
     </row>
@@ -3372,7 +3512,7 @@
     <row r="72" ht="15.75" customHeight="1" s="109">
       <c r="A72" s="110" t="inlineStr">
         <is>
-          <t>4. BAS - Sep quarter (Sep PAYG ~$50k + GST est ~$50k + any instalment) is due 28 Oct as we lodge it ourselves - it's in week 4. Swap the GST estimate for the activity statement figure once it's run.</t>
+          <t>4. BAS - Sep quarter (~$96k) did not go out on 28 Oct. Confirm whether it is lodged through the agent (25 Nov) - it is in the 29 Oct forecast on that date. Swap the GST estimate for the activity statement figure.</t>
         </is>
       </c>
     </row>

</xml_diff>